<commit_message>
Update Lembar Coding Fenny dan Kunci Adjukasi
</commit_message>
<xml_diff>
--- a/P4 Pengembangan Kebutuhan Perangkat Lunak/A Elisitasi/A4 Coding/20261027 Lembar_Coding_Codebook_1_0_3 (Afriansyah).xlsx
+++ b/P4 Pengembangan Kebutuhan Perangkat Lunak/A Elisitasi/A4 Coding/20261027 Lembar_Coding_Codebook_1_0_3 (Afriansyah).xlsx
@@ -6605,7 +6605,7 @@
     </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="8" disablePrompts="0">
-        <x14:dataValidation xr:uid="{6B446CB6-EDB9-4C3B-AB38-29A1613E072D}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Kodekan pihak yang secara eksplisit menjadi subjek tata bahasa norma utama pada kolom “Isi”.&#10;Pilih kode berurutan dan berhenti pada Subjek Norma pertama yang dianggap sesuai (S1 &gt; S2 &gt; S3 &gt; S4 &gt; S5 &gt; S6 &gt; S7 &gt; S8 &gt; S9)." showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{5AB987B5-8F3F-4A18-8FCD-1A01250F3F1E}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Kodekan pihak yang secara eksplisit menjadi subjek tata bahasa norma utama pada kolom “Isi”.&#10;Pilih kode berurutan dan berhenti pada Subjek Norma pertama yang dianggap sesuai (S1 &gt; S2 &gt; S3 &gt; S4 &gt; S5 &gt; S6 &gt; S7 &gt; S8 &gt; S9)." showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>'Daftar Kode'!$D$5:$D$13</xm:f>
           </x14:formula1>
@@ -6614,7 +6614,7 @@
           </x14:formula2>
           <xm:sqref>F3:F86</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{40B5306A-ACA4-44F8-869E-4F684B7016F6}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Tentukan dengan Uji Implikasi Bagian 6." promptTitle="" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{6956030B-6D2B-46A8-B5E5-A9E353C50442}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Tentukan dengan Uji Implikasi Bagian 6." promptTitle="" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>'Daftar Kode'!$D$16:$D$18</xm:f>
           </x14:formula1>
@@ -6623,7 +6623,7 @@
           </x14:formula2>
           <xm:sqref>G2:G86</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{732788A8-FF50-46FF-988A-701FEA389DEA}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Pilih satu tema dominan dari pohon keputusan Bagian 7.3. Pemilihan T99 wajib dijelaskan di V12." showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{0235AB53-B601-4F0C-A78B-81CF67D714A8}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Pilih satu tema dominan dari pohon keputusan Bagian 7.3. Pemilihan T99 wajib dijelaskan di V12." showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>'Daftar Kode'!$D$21:$D$37</xm:f>
           </x14:formula1>
@@ -6632,7 +6632,7 @@
           </x14:formula2>
           <xm:sqref>H2:H86</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{7B9CE856-6B53-41A3-A492-8CCC33ED0A3A}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Lihat Bagian 7.4" promptTitle="" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{4D785A3B-70C9-48E7-9453-970154BC1193}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Lihat Bagian 7.4" promptTitle="" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>'Daftar Kode'!$D$40:$D$47</xm:f>
           </x14:formula1>
@@ -6641,7 +6641,7 @@
           </x14:formula2>
           <xm:sqref>I2:I86</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{3E6C701A-4875-42DE-A512-132E7B5E9E91}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Tahap siklus data yang terkait dari awal hingga akhir.&#10;Lihat Bagian 7.5" promptTitle="" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{2C13D2DA-D41C-41BE-A982-016866542D6A}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Tahap siklus data yang terkait dari awal hingga akhir.&#10;Lihat Bagian 7.5" promptTitle="" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>'Daftar Kode'!$D$50:$D$57</xm:f>
           </x14:formula1>
@@ -6650,7 +6650,7 @@
           </x14:formula2>
           <xm:sqref>J2:J86</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{3279EF55-5946-4DE2-9654-D05273BA8A11}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Kandidat jenis kebutuhan SRS diperiksa berurutan K1 &gt; K2 &gt; K3 &gt; K4 &gt; K5. Lihat Bagian 7.6" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{2B5F0096-AB80-4B6C-9FA2-0BED7272C486}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Kandidat jenis kebutuhan SRS diperiksa berurutan K1 &gt; K2 &gt; K3 &gt; K4 &gt; K5. Lihat Bagian 7.6" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>'Daftar Kode'!$D$60:$D$64</xm:f>
           </x14:formula1>
@@ -6659,7 +6659,7 @@
           </x14:formula2>
           <xm:sqref>K2:K86</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{213DA5A4-8CE0-4364-A748-72F014A5DE1F}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Tema kedua bila unit memuat dua tema (gunakan kode dari Bagian 7.3). T99 tidak digunakan di sini." promptTitle="Opsional" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{65DDCB1A-04FF-4B4F-B401-52E603A7A314}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Tema kedua bila unit memuat dua tema (gunakan kode dari Bagian 7.3). T99 tidak digunakan di sini." promptTitle="Opsional" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>'Daftar Kode'!$D$21:$D$36</xm:f>
           </x14:formula1>
@@ -6668,7 +6668,7 @@
           </x14:formula2>
           <xm:sqref>L2:L86</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{7170DCE0-C8F8-4E94-BFBE-0BA7EC86068A}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Kodekan pihak yang secara eksplisit menjadi subjek tata bahasa norma utama pada kolom “Isi”. Jangan menyimpulkan subjek dari judul BAB." showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{2129703A-C87D-4D30-91F9-00316166868E}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Kodekan pihak yang secara eksplisit menjadi subjek tata bahasa norma utama pada kolom “Isi”. Jangan menyimpulkan subjek dari judul BAB." showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>'Daftar Kode'!$D$5:$D$13</xm:f>
           </x14:formula1>

</xml_diff>

<commit_message>
Hasil pilot Fenny, Deni, Afriansyah
</commit_message>
<xml_diff>
--- a/P4 Pengembangan Kebutuhan Perangkat Lunak/A Elisitasi/A4 Coding/20261027 Lembar_Coding_Codebook_1_0_3 (Afriansyah).xlsx
+++ b/P4 Pengembangan Kebutuhan Perangkat Lunak/A Elisitasi/A4 Coding/20261027 Lembar_Coding_Codebook_1_0_3 (Afriansyah).xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="402" uniqueCount="402">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="408">
   <si>
     <t xml:space="preserve">Lembar Coding: Analisis Isi Krippendorff</t>
   </si>
@@ -211,6 +211,27 @@
     <t>Bagian</t>
   </si>
   <si>
+    <t xml:space="preserve">S9 - Tidak ada subjek perorangan atau organisasi eksplisit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R2 - Relevan langsung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T11 - Keamanan, Kerahasiaan, dan Penanganan Insiden</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P7 - Asas, prinsip, atau tujuan umum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F8 - Lintas tahap atau tidak spesifik</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K1 - Non-fungsional: keamanan dan kerahasiaan. Apakah inti teks melindungi data dari akses atau gangguan tidak sah?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T03 - Larangan dan Perbuatan Melawan Hukum</t>
+  </si>
+  <si>
     <t>CC</t>
   </si>
   <si>
@@ -229,9 +250,6 @@
     <t xml:space="preserve">F7 - Tata kelola dan hak subjek</t>
   </si>
   <si>
-    <t xml:space="preserve">K1 - Non-fungsional: keamanan dan kerahasiaan. Apakah inti teks melindungi data dari akses atau gangguan tidak sah?</t>
-  </si>
-  <si>
     <t xml:space="preserve">T15 - Asas dan Prinsip Pemrosesan</t>
   </si>
   <si>
@@ -241,16 +259,25 @@
     <t>Ya</t>
   </si>
   <si>
+    <t xml:space="preserve">T02 - Latar Normatif dan Rujukan Non-operasional</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P8 - Deskriptif, argumentatif, dan rujukan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K2 - Non-fungsional: mutu data, kepatuhan, dan akuntabilitas. Apakah ini mutu atau bukti yang berlaku untuk seluruh sistem, bukan hanya satu operasi?</t>
+  </si>
+  <si>
     <t xml:space="preserve">S7 - Otoritas Penetap atau Pengawas Kebijakan</t>
   </si>
   <si>
-    <t xml:space="preserve">T02 - Latar Normatif dan Rujukan Non-operasional</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P8 - Deskriptif, argumentatif, dan rujukan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">K2 - Non-fungsional: mutu data, kepatuhan, dan akuntabilitas. Apakah ini mutu atau bukti yang berlaku untuk seluruh sistem, bukan hanya satu operasi?</t>
+    <t xml:space="preserve">S8 - Penyelenggara sektor atau pihak lain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P2 - Kewajiban</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T08 - Retensi, Penghentian, Penghapusan, dan Pemusnahan</t>
   </si>
   <si>
     <t xml:space="preserve">R0 - Tidak relevan</t>
@@ -259,76 +286,58 @@
     <t xml:space="preserve">K5 - Tidak menghasilkan kebutuhan. Apakah teks benar-benar tidak dapat diterjemahkan menjadi kalimat "Sistem harus/tidak boleh …"?</t>
   </si>
   <si>
-    <t xml:space="preserve">T11 - Keamanan, Kerahasiaan, dan Penanganan Insiden</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S9 - Tidak ada subjek perorangan atau organisasi eksplisit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P7 - Asas, prinsip, atau tujuan umum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F8 - Lintas tahap atau tidak spesifik</t>
+    <t xml:space="preserve">P6 - Definisi, klasifikasi, atau ruang lingkup</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K4 - Batasan atau aturan bisnis hukum. Apakah teks membatasi apa yang boleh dilakukan sistem, atau apa dan siapa yang tercakup?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T05 - Jenis dan Klasifikasi Data Pribadi</t>
   </si>
   <si>
     <t xml:space="preserve">T13 - Akuntabilitas, Pencatatan, dan Tata Kelola Kepatuhan</t>
   </si>
   <si>
-    <t xml:space="preserve">R2 - Relevan langsung</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T08 - Retensi, Penghentian, Penghapusan, dan Pemusnahan</t>
+    <t xml:space="preserve">T07 - Hak Subjek Data Pribadi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K3 - Fungsional. Dapatkah ditulis "Sistem harus [melakukan X]" dengan hasil hanya lulus atau gagal?</t>
   </si>
   <si>
     <t xml:space="preserve">F6 - Retensi dan penghapusan</t>
   </si>
   <si>
-    <t xml:space="preserve">K3 - Fungsional. Dapatkah ditulis "Sistem harus [melakukan X]" dengan hasil hanya lulus atau gagal?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T07 - Hak Subjek Data Pribadi</t>
-  </si>
-  <si>
     <t xml:space="preserve">T04 - Pengecualian dan Pembatasan</t>
   </si>
   <si>
-    <t xml:space="preserve">K4 - Batasan atau aturan bisnis hukum. Apakah teks membatasi apa yang boleh dilakukan sistem, atau apa dan siapa yang tercakup?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S8 - Penyelenggara sektor atau pihak lain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P6 - Definisi, klasifikasi, atau ruang lingkup</t>
-  </si>
-  <si>
     <t xml:space="preserve">F2 - Pengumpulan atau akuisisi</t>
   </si>
   <si>
     <t xml:space="preserve">T16 - Aktivitas Pemrosesan dan Pengumpulan</t>
   </si>
   <si>
+    <t xml:space="preserve">T09 - Dasar Pemrosesan dan Persetujuan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F1 - Perencanaan dan dasar pemrosesan</t>
+  </si>
+  <si>
     <t xml:space="preserve">S5 - Setiap Orang atau pihak umum</t>
   </si>
   <si>
     <t xml:space="preserve">T06 - Data Pribadi Anak dan Kelompok Rentan</t>
   </si>
   <si>
-    <t xml:space="preserve">P2 - Kewajiban</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T09 - Dasar Pemrosesan dan Persetujuan</t>
-  </si>
-  <si>
     <t xml:space="preserve">S2 - Pengendali Data Pribadi</t>
   </si>
   <si>
-    <t xml:space="preserve">F1 - Perencanaan dan dasar pemrosesan</t>
+    <t xml:space="preserve">F3 - Pengolahan dan analisis</t>
   </si>
   <si>
     <t xml:space="preserve">T12 - Kualitas, Akurasi, dan Pembaruan Data</t>
   </si>
   <si>
-    <t xml:space="preserve">F3 - Pengolahan dan analisis</t>
+    <t xml:space="preserve">F4 - Penyimpanan dan pengamanan</t>
   </si>
   <si>
     <t xml:space="preserve">T10 - Transfer dan Pengalihan Data</t>
@@ -338,6 +347,15 @@
   </si>
   <si>
     <t xml:space="preserve">F5 - Penyebarluasan dan transfer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P1 - Larangan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S6 - Instansi atau Badan Publik</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T14 - Akses dan Pemanfaatan Data Pemerintah</t>
   </si>
   <si>
     <t xml:space="preserve">Daftar kode sah (Codebook versi 1.0.3)</t>
@@ -2245,25 +2263,39 @@
         <f>IF(INDEX(Korpus!$F:$F,$A2)="","",INDEX(Korpus!$F:$F,$A2))</f>
         <v xml:space="preserve">Melihat banyaknya kasus penyalahgunaan data pribadi, sangat penting untuk memberikan perlindungan data pribadi.</v>
       </c>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
-      <c r="H2" s="18"/>
-      <c r="I2" s="18"/>
-      <c r="J2" s="18"/>
-      <c r="K2" s="18"/>
-      <c r="L2" s="18"/>
+      <c r="F2" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="G2" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="H2" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="I2" s="18" t="s">
+        <v>65</v>
+      </c>
+      <c r="J2" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="K2" s="18" t="s">
+        <v>67</v>
+      </c>
+      <c r="L2" s="18" t="s">
+        <v>68</v>
+      </c>
       <c r="M2" s="19"/>
       <c r="N2" s="19"/>
       <c r="O2" s="15" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="P2" s="17" t="str">
         <f t="shared" ref="P2:P9" si="0">IF(COUNTA(F2:K2)=6,"Lengkap","Belum lengkap ("&amp;(6-COUNTA(F2:K2))&amp;")")</f>
-        <v xml:space="preserve">Belum lengkap (6)</v>
+        <v>Lengkap</v>
       </c>
       <c r="Q2" s="17" t="str">
         <f t="shared" ref="Q2:Q9" si="1">IF(COUNTA(F2:K2)&lt;6,"",IF(IF(AND(LEFT(G2,2)="R0",LEFT(K2,2)&lt;&gt;"K5"),"R0 harus K5; ","")&amp;IF(AND(LEFT(G2,2)="R1",LEFT(K2,2)="K3"),"R1 tidak boleh K3 (fungsional); ","")&amp;IF(AND(LEFT(G2,2)="R2",LEFT(K2,2)="K5"),"R2 tidak boleh K5; ","")&amp;IF(AND(LEFT(G2,2)="R2",OR(LEFT(F2,2)="S6",LEFT(F2,2)="S7",LEFT(F2,2)="S8")),"R2 tidak boleh S6/S7/S8; ","")&amp;IF(AND(LEFT(G2,2)="R2",OR(LEFT(H2,3)="T02",LEFT(I2,2)="P8")),"T02 atau P8 tidak boleh R2; ","")&amp;IF(AND(LEFT(H2,3)="T01",LEFT(I2,2)&lt;&gt;"P6",N2=""),"T01 biasanya P6; jelaskan di V12; ","")&amp;IF(AND(LEFT(I2,2)="P1",LEFT(K2,2)&lt;&gt;"K4",N2=""),"P1 biasanya K4; jelaskan di V12; ","")="","OK",IF(AND(LEFT(G2,2)="R0",LEFT(K2,2)&lt;&gt;"K5"),"R0 harus K5; ","")&amp;IF(AND(LEFT(G2,2)="R1",LEFT(K2,2)="K3"),"R1 tidak boleh K3 (fungsional); ","")&amp;IF(AND(LEFT(G2,2)="R2",LEFT(K2,2)="K5"),"R2 tidak boleh K5; ","")&amp;IF(AND(LEFT(G2,2)="R2",OR(LEFT(F2,2)="S6",LEFT(F2,2)="S7",LEFT(F2,2)="S8")),"R2 tidak boleh S6/S7/S8; ","")&amp;IF(AND(LEFT(G2,2)="R2",OR(LEFT(H2,3)="T02",LEFT(I2,2)="P8")),"T02 atau P8 tidak boleh R2; ","")&amp;IF(AND(LEFT(H2,3)="T01",LEFT(I2,2)&lt;&gt;"P6",N2=""),"T01 biasanya P6; jelaskan di V12; ","")&amp;IF(AND(LEFT(I2,2)="P1",LEFT(K2,2)&lt;&gt;"K4",N2=""),"P1 biasanya K4; jelaskan di V12; ","")))</f>
-        <v/>
+        <v>OK</v>
       </c>
       <c r="R2" s="17" t="str">
         <f>IF(INDEX(Korpus!$B:$B,$A2)="","",INDEX(Korpus!$B:$B,$A2))</f>
@@ -2274,7 +2306,7 @@
         <v xml:space="preserve">5. Pentingnya Perlindungan Data Pribadi</v>
       </c>
     </row>
-    <row r="3" ht="60" hidden="1" customHeight="1">
+    <row r="3" ht="60" customHeight="1">
       <c r="A3" s="15">
         <v>3</v>
       </c>
@@ -2321,7 +2353,7 @@
         <v xml:space="preserve">5. Pentingnya Perlindungan Data Pribadi</v>
       </c>
     </row>
-    <row r="4" ht="60" hidden="1" customHeight="1">
+    <row r="4" ht="60" customHeight="1">
       <c r="A4" s="15">
         <v>4</v>
       </c>
@@ -2368,7 +2400,7 @@
         <v xml:space="preserve">5. Pentingnya Perlindungan Data Pribadi</v>
       </c>
     </row>
-    <row r="5" ht="60" hidden="1" customHeight="1">
+    <row r="5" ht="60" customHeight="1">
       <c r="A5" s="15">
         <v>5</v>
       </c>
@@ -2415,7 +2447,7 @@
         <v xml:space="preserve">5. Pentingnya Perlindungan Data Pribadi</v>
       </c>
     </row>
-    <row r="6" ht="60" hidden="1" customHeight="1">
+    <row r="6" ht="60" customHeight="1">
       <c r="A6" s="15">
         <v>6</v>
       </c>
@@ -2462,7 +2494,7 @@
         <v xml:space="preserve">5. Pentingnya Perlindungan Data Pribadi</v>
       </c>
     </row>
-    <row r="7" ht="60" hidden="1" customHeight="1">
+    <row r="7" ht="60" customHeight="1">
       <c r="A7" s="15">
         <v>7</v>
       </c>
@@ -2509,7 +2541,7 @@
         <v xml:space="preserve">5. Pentingnya Perlindungan Data Pribadi</v>
       </c>
     </row>
-    <row r="8" ht="60" hidden="1" customHeight="1">
+    <row r="8" ht="60" customHeight="1">
       <c r="A8" s="15">
         <v>8</v>
       </c>
@@ -2556,7 +2588,7 @@
         <v xml:space="preserve">5. Pentingnya Perlindungan Data Pribadi</v>
       </c>
     </row>
-    <row r="9" ht="60" hidden="1" customHeight="1">
+    <row r="9" ht="60" customHeight="1">
       <c r="A9" s="15">
         <v>9</v>
       </c>
@@ -2603,7 +2635,7 @@
         <v xml:space="preserve">5. Pentingnya Perlindungan Data Pribadi</v>
       </c>
     </row>
-    <row r="10" ht="60" hidden="1" customHeight="1">
+    <row r="10" ht="60" customHeight="1">
       <c r="A10" s="15">
         <v>10</v>
       </c>
@@ -2650,7 +2682,7 @@
         <v xml:space="preserve">5. Pentingnya Perlindungan Data Pribadi</v>
       </c>
     </row>
-    <row r="11" ht="60" hidden="1" customHeight="1">
+    <row r="11" ht="60" customHeight="1">
       <c r="A11" s="15">
         <v>11</v>
       </c>
@@ -2697,7 +2729,7 @@
         <v xml:space="preserve">5. Pentingnya Perlindungan Data Pribadi</v>
       </c>
     </row>
-    <row r="12" ht="60" hidden="1" customHeight="1">
+    <row r="12" ht="60" customHeight="1">
       <c r="A12" s="15">
         <v>12</v>
       </c>
@@ -2744,7 +2776,7 @@
         <v xml:space="preserve">5. Pentingnya Perlindungan Data Pribadi</v>
       </c>
     </row>
-    <row r="13" ht="60" hidden="1" customHeight="1">
+    <row r="13" ht="60" customHeight="1">
       <c r="A13" s="15">
         <v>13</v>
       </c>
@@ -2765,32 +2797,32 @@
         <v xml:space="preserve">Dalam Pasal 28 G ayat (1) disebutkan bahwa “Setiap orang berhak atas perlindungan diri pribadi, data juga berhubungan dengan konsep hak keluarga, kehormatan, martabat, dan harta benda yang di bawah kekuasaannya, serta berhak atas rasa aman dan perlindungan dari ancaman ketakutan untuk berbuat atau tidak berbuat sesuatu yang merupakan hak asasi.”</v>
       </c>
       <c r="F13" s="18" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="G13" s="18" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="H13" s="18" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="I13" s="18" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="J13" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="K13" s="18" t="s">
         <v>67</v>
       </c>
-      <c r="K13" s="18" t="s">
-        <v>68</v>
-      </c>
       <c r="L13" s="18" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="M13" s="19"/>
       <c r="N13" s="19" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="O13" s="15" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="P13" s="17" t="str">
         <f t="shared" si="2"/>
@@ -2809,7 +2841,7 @@
         <v xml:space="preserve">5. Pentingnya Perlindungan Data Pribadi</v>
       </c>
     </row>
-    <row r="14" ht="60" hidden="1" customHeight="1">
+    <row r="14" ht="60" customHeight="1">
       <c r="A14" s="15">
         <v>14</v>
       </c>
@@ -2876,25 +2908,39 @@
         <f>IF(INDEX(Korpus!$F:$F,$A15)="","",INDEX(Korpus!$F:$F,$A15))</f>
         <v xml:space="preserve">1) Undang-Undang Nomor 19 Tahun 2016 Tentang Perubahan Atas Undang-Undang Nomor 11 Tahun 2008 Tentang Informasi dan Transaksi Elektronik</v>
       </c>
-      <c r="F15" s="18"/>
-      <c r="G15" s="18"/>
-      <c r="H15" s="18"/>
-      <c r="I15" s="18"/>
-      <c r="J15" s="18"/>
-      <c r="K15" s="18"/>
-      <c r="L15" s="18"/>
+      <c r="F15" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="G15" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="H15" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="I15" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="J15" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="K15" s="18" t="s">
+        <v>80</v>
+      </c>
+      <c r="L15" s="18" t="s">
+        <v>64</v>
+      </c>
       <c r="M15" s="19"/>
       <c r="N15" s="19"/>
       <c r="O15" s="15" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="P15" s="17" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve">Belum lengkap (6)</v>
+        <v>Lengkap</v>
       </c>
       <c r="Q15" s="17" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>OK</v>
       </c>
       <c r="R15" s="17" t="str">
         <f>IF(INDEX(Korpus!$B:$B,$A15)="","",INDEX(Korpus!$B:$B,$A15))</f>
@@ -2905,7 +2951,7 @@
         <v xml:space="preserve">5. Pentingnya Perlindungan Data Pribadi</v>
       </c>
     </row>
-    <row r="16" ht="60" hidden="1" customHeight="1">
+    <row r="16" ht="60" customHeight="1">
       <c r="A16" s="15">
         <v>16</v>
       </c>
@@ -2952,7 +2998,7 @@
         <v xml:space="preserve">5. Pentingnya Perlindungan Data Pribadi</v>
       </c>
     </row>
-    <row r="17" ht="60" hidden="1" customHeight="1">
+    <row r="17" ht="60" customHeight="1">
       <c r="A17" s="15">
         <v>17</v>
       </c>
@@ -2999,7 +3045,7 @@
         <v xml:space="preserve">5. Pentingnya Perlindungan Data Pribadi</v>
       </c>
     </row>
-    <row r="18" ht="60" hidden="1" customHeight="1">
+    <row r="18" ht="60" customHeight="1">
       <c r="A18" s="15">
         <v>18</v>
       </c>
@@ -3046,7 +3092,7 @@
         <v xml:space="preserve">5. Pentingnya Perlindungan Data Pribadi</v>
       </c>
     </row>
-    <row r="19" ht="60" hidden="1" customHeight="1">
+    <row r="19" ht="60" customHeight="1">
       <c r="A19" s="15">
         <v>19</v>
       </c>
@@ -3093,7 +3139,7 @@
         <v xml:space="preserve">5. Pentingnya Perlindungan Data Pribadi</v>
       </c>
     </row>
-    <row r="20" ht="60" hidden="1" customHeight="1">
+    <row r="20" ht="60" customHeight="1">
       <c r="A20" s="15">
         <v>20</v>
       </c>
@@ -3140,7 +3186,7 @@
         <v xml:space="preserve">5. Pentingnya Perlindungan Data Pribadi</v>
       </c>
     </row>
-    <row r="21" ht="60" hidden="1" customHeight="1">
+    <row r="21" ht="60" customHeight="1">
       <c r="A21" s="15">
         <v>21</v>
       </c>
@@ -3161,30 +3207,30 @@
         <v xml:space="preserve">Selain itu Peraturan OJK Nomor 13 Tahun 2018 Tentang Inovasi Keuangan Digital di Sektor Keuangan, telah memasukkan poin terkait perlindungan dan kerahasiaan data.</v>
       </c>
       <c r="F21" s="18" t="s">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="G21" s="18" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="H21" s="18" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="I21" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="J21" s="18" t="s">
         <v>74</v>
       </c>
-      <c r="J21" s="18" t="s">
-        <v>67</v>
-      </c>
       <c r="K21" s="18" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="L21" s="18" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="M21" s="19"/>
       <c r="N21" s="19"/>
       <c r="O21" s="15" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="P21" s="17" t="str">
         <f t="shared" si="2"/>
@@ -3223,25 +3269,39 @@
         <f>IF(INDEX(Korpus!$F:$F,$A22)="","",INDEX(Korpus!$F:$F,$A22))</f>
         <v xml:space="preserve">Pasal 30 ayat (1) menyebutkan bahwa Penyelenggara wajib menjaga kerahasiaan data pribadi, data transaksi, dan data keuangan yang dikelolanya sejak diperoleh hingga data tersebut dimusnahkan.</v>
       </c>
-      <c r="F22" s="18"/>
-      <c r="G22" s="18"/>
-      <c r="H22" s="18"/>
-      <c r="I22" s="18"/>
-      <c r="J22" s="18"/>
-      <c r="K22" s="18"/>
-      <c r="L22" s="18"/>
+      <c r="F22" s="18" t="s">
+        <v>82</v>
+      </c>
+      <c r="G22" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="H22" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="I22" s="18" t="s">
+        <v>83</v>
+      </c>
+      <c r="J22" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="K22" s="18" t="s">
+        <v>67</v>
+      </c>
+      <c r="L22" s="18" t="s">
+        <v>84</v>
+      </c>
       <c r="M22" s="19"/>
       <c r="N22" s="19"/>
       <c r="O22" s="15" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="P22" s="17" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve">Belum lengkap (6)</v>
+        <v>Lengkap</v>
       </c>
       <c r="Q22" s="17" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>OK</v>
       </c>
       <c r="R22" s="17" t="str">
         <f>IF(INDEX(Korpus!$B:$B,$A22)="","",INDEX(Korpus!$B:$B,$A22))</f>
@@ -3252,7 +3312,7 @@
         <v xml:space="preserve">5. Pentingnya Perlindungan Data Pribadi</v>
       </c>
     </row>
-    <row r="23" ht="60" hidden="1" customHeight="1">
+    <row r="23" ht="60" customHeight="1">
       <c r="A23" s="15">
         <v>23</v>
       </c>
@@ -3299,7 +3359,7 @@
         <v xml:space="preserve">5. Pentingnya Perlindungan Data Pribadi</v>
       </c>
     </row>
-    <row r="24" ht="60" hidden="1" customHeight="1">
+    <row r="24" ht="60" customHeight="1">
       <c r="A24" s="15">
         <v>24</v>
       </c>
@@ -3346,7 +3406,7 @@
         <v xml:space="preserve">5. Pentingnya Perlindungan Data Pribadi</v>
       </c>
     </row>
-    <row r="25" ht="60" hidden="1" customHeight="1">
+    <row r="25" ht="60" customHeight="1">
       <c r="A25" s="15">
         <v>25</v>
       </c>
@@ -3367,30 +3427,30 @@
         <v xml:space="preserve">Selain itu juga sudah ada Peraturan Menteri Nomor 20 Tahun 2016 tentang Perlindungan Data Pribadi namun belum cukup memberikan perlindungan kepada konsumen.</v>
       </c>
       <c r="F25" s="18" t="s">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="G25" s="18" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
       <c r="H25" s="18" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="I25" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="J25" s="18" t="s">
         <v>74</v>
       </c>
-      <c r="J25" s="18" t="s">
-        <v>67</v>
-      </c>
       <c r="K25" s="18" t="s">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="L25" s="18" t="s">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="M25" s="19"/>
       <c r="N25" s="19"/>
       <c r="O25" s="15" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="P25" s="17" t="str">
         <f t="shared" si="2"/>
@@ -3409,7 +3469,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" ht="60" hidden="1" customHeight="1">
+    <row r="26" ht="60" customHeight="1">
       <c r="A26" s="15">
         <v>26</v>
       </c>
@@ -3456,7 +3516,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" ht="60" hidden="1" customHeight="1">
+    <row r="27" ht="60" customHeight="1">
       <c r="A27" s="15">
         <v>27</v>
       </c>
@@ -3505,7 +3565,7 @@
 Identitas Anak</v>
       </c>
     </row>
-    <row r="28" ht="60" customHeight="1">
+    <row r="28" ht="395.25">
       <c r="A28" s="15">
         <v>28</v>
       </c>
@@ -3525,25 +3585,39 @@
         <f>IF(INDEX(Korpus!$F:$F,$A28)="","",INDEX(Korpus!$F:$F,$A28))</f>
         <v xml:space="preserve">Dalam Undang-Undang ini yang dimaksud dengan: 1. Data Pribadi adalah data tentang orang perseorangan yang teridentifikasi atau dapat diidentifikasi secara tersendiri atau dikombinasi dengan informasi lainnya baik secara langsung maupun tidak langsung melalui sistem elektronik atau nonelektronik. 2. Pelindungan Data Pribadi adalah keseluruhan upaya untuk melindungi Data Pribadi dalam rangkaian pemrosesan Data Pribadi guna menjamin hak konstitusional subjek Data Pribadi. 3. Informasi adalah keterangan, pernyataan, gagasan, dan tanda-tanda yang mengandung nilai, makna, dan pesan, baik data, fakta, maupun penjelasannya yang dapat dilihat, didengar, dan dibaca yang disajikan dalam berbagai kemasan dan format sesuai dengan perkembangan teknologi informasi dan komunikasi secara elektronik ataupun nonelektronik. 4. Pengendali Data Pribadi adalah setiap orang, badan publik, dan organisasi internasional yang bertindak sendiri-sendiri atau bersama-sama dalam menentukan tujuan dan melakukan kendali pemrosesan Data Pribadi. 5. Prosesor Data Pribadi adalah setiap orang, badan publik, dan organisasi internasional yang bertindak sendiri-sendiri atau bersama-sama dalam melakukan pemrosesan Data Pribadi atas nama Pengendali Data Pribadi. 6. Subjek Data Pribadi adalah orang perseorangan yang pada dirinya melekat Data Pribadi. 7. Setiap Orang adalah orang perseorangan atau korporasi. 8. Korporasi adalah kumpulan orang dan/ atau kekayaan yang terorganisasi baik yang berbadan hukum maupun tidak berbadan hukum. 9. Badan Publik adalah lembaga eksekutif, legislatif, yudikatif, dan badan lain yang fungsi dan tugas pokoknya berkaitan dengan penyelenggaraan negara, yang sebagian atau seluruh dananya bersumber dari Anggaran Pendapatan dan Belanja Negara dan/ atau Anggaran Pendapatan dan Belanja Daerah, atau organisasi nonpemerintah sepanjang sebagian atau seluruh dananya bersumber dari Anggaran Pendapatan dan Belanja Negara dan/ atau Anggaran. Pendapatan dan Belanja Daerah, sumbangan masyarakat, dan/atau luar negeri. 10. Organisasi Internasional adalah organisasi yang diakui sebagai subjek hukum internasional dan mempunyai kapasitas untuk membuat perjanjian internasional.</v>
       </c>
-      <c r="F28" s="18"/>
-      <c r="G28" s="18"/>
-      <c r="H28" s="18"/>
-      <c r="I28" s="18"/>
-      <c r="J28" s="18"/>
-      <c r="K28" s="18"/>
-      <c r="L28" s="18"/>
+      <c r="F28" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="G28" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="H28" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="I28" s="18" t="s">
+        <v>87</v>
+      </c>
+      <c r="J28" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="K28" s="18" t="s">
+        <v>88</v>
+      </c>
+      <c r="L28" s="18" t="s">
+        <v>89</v>
+      </c>
       <c r="M28" s="19"/>
       <c r="N28" s="19"/>
       <c r="O28" s="15" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="P28" s="17" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve">Belum lengkap (6)</v>
+        <v>Lengkap</v>
       </c>
       <c r="Q28" s="17" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>OK</v>
       </c>
       <c r="R28" s="17" t="str">
         <f>IF(INDEX(Korpus!$B:$B,$A28)="","",INDEX(Korpus!$B:$B,$A28))</f>
@@ -3555,7 +3629,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" ht="60" hidden="1" customHeight="1">
+    <row r="29" ht="60" customHeight="1">
       <c r="A29" s="15">
         <v>29</v>
       </c>
@@ -3603,7 +3677,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" ht="60" hidden="1" customHeight="1">
+    <row r="30" ht="60" customHeight="1">
       <c r="A30" s="15">
         <v>30</v>
       </c>
@@ -3624,30 +3698,30 @@
         <v xml:space="preserve">a. perlindungan; b. kepastian hukum; c. kepentingan umum; d. Kemanfaatan; e. Kehati-hatian; f. Keseimbangan; g. Pertanggungjawaban; dan h. kerahasiaan.</v>
       </c>
       <c r="F30" s="18" t="s">
-        <v>79</v>
+        <v>62</v>
       </c>
       <c r="G30" s="18" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
       <c r="H30" s="18" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="I30" s="18" t="s">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="J30" s="18" t="s">
-        <v>81</v>
+        <v>66</v>
       </c>
       <c r="K30" s="18" t="s">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="L30" s="18" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="M30" s="19"/>
       <c r="N30" s="19"/>
       <c r="O30" s="15" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="P30" s="17" t="str">
         <f t="shared" si="2"/>
@@ -3667,7 +3741,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" ht="60" hidden="1" customHeight="1">
+    <row r="31" ht="60" customHeight="1">
       <c r="A31" s="15">
         <v>31</v>
       </c>
@@ -3735,25 +3809,39 @@
         <f>IF(INDEX(Korpus!$F:$F,$A32)="","",INDEX(Korpus!$F:$F,$A32))</f>
         <v xml:space="preserve">Subjek Data Pribadi berhak mendapatkan Informasi tentang kejelasan identitas, dasar kepentingan hukum, tujuan permintaan dan penggunaan Data Pribadi, dan akuntabilitas pihak yang meminta Data Pribadi.</v>
       </c>
-      <c r="F32" s="18"/>
-      <c r="G32" s="18"/>
-      <c r="H32" s="18"/>
-      <c r="I32" s="18"/>
-      <c r="J32" s="18"/>
-      <c r="K32" s="18"/>
-      <c r="L32" s="18"/>
+      <c r="F32" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="G32" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="H32" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="I32" s="18" t="s">
+        <v>73</v>
+      </c>
+      <c r="J32" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="K32" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="L32" s="18" t="s">
+        <v>90</v>
+      </c>
       <c r="M32" s="19"/>
       <c r="N32" s="19"/>
       <c r="O32" s="15" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="P32" s="17" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve">Belum lengkap (6)</v>
+        <v>Lengkap</v>
       </c>
       <c r="Q32" s="17" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>OK</v>
       </c>
       <c r="R32" s="17" t="str">
         <f>IF(INDEX(Korpus!$B:$B,$A32)="","",INDEX(Korpus!$B:$B,$A32))</f>
@@ -3765,7 +3853,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" ht="60" hidden="1" customHeight="1">
+    <row r="33" ht="60" customHeight="1">
       <c r="A33" s="15">
         <v>33</v>
       </c>
@@ -3813,7 +3901,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" ht="60" hidden="1" customHeight="1">
+    <row r="34" ht="60" customHeight="1">
       <c r="A34" s="15">
         <v>34</v>
       </c>
@@ -3861,7 +3949,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" ht="60" hidden="1" customHeight="1">
+    <row r="35" ht="60" customHeight="1">
       <c r="A35" s="15">
         <v>35</v>
       </c>
@@ -3882,30 +3970,30 @@
         <v xml:space="preserve">Subjek Data Pribadi berhak untuk mengakhiri pemrosesan, menghapus, dan/ atau memusnahkan Data Pribadi tentang dirinya sesuai dengan ketentuan peraturan perundang-undangan.</v>
       </c>
       <c r="F35" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="G35" s="18" t="s">
         <v>63</v>
-      </c>
-      <c r="G35" s="18" t="s">
-        <v>83</v>
       </c>
       <c r="H35" s="18" t="s">
         <v>84</v>
       </c>
       <c r="I35" s="18" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="J35" s="18" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="K35" s="18" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="L35" s="18" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="M35" s="19"/>
       <c r="N35" s="19"/>
       <c r="O35" s="15" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="P35" s="17" t="str">
         <f t="shared" si="2"/>
@@ -3925,7 +4013,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" ht="60" hidden="1" customHeight="1">
+    <row r="36" ht="60" customHeight="1">
       <c r="A36" s="15">
         <v>36</v>
       </c>
@@ -3973,7 +4061,7 @@
         <v/>
       </c>
     </row>
-    <row r="37" ht="60" hidden="1" customHeight="1">
+    <row r="37" ht="60" customHeight="1">
       <c r="A37" s="15">
         <v>37</v>
       </c>
@@ -4021,7 +4109,7 @@
         <v/>
       </c>
     </row>
-    <row r="38" ht="60" hidden="1" customHeight="1">
+    <row r="38" ht="60" customHeight="1">
       <c r="A38" s="15">
         <v>38</v>
       </c>
@@ -4069,7 +4157,7 @@
         <v/>
       </c>
     </row>
-    <row r="39" ht="60" hidden="1" customHeight="1">
+    <row r="39" ht="60" customHeight="1">
       <c r="A39" s="15">
         <v>39</v>
       </c>
@@ -4117,7 +4205,7 @@
         <v/>
       </c>
     </row>
-    <row r="40" ht="60" hidden="1" customHeight="1">
+    <row r="40" ht="60" customHeight="1">
       <c r="A40" s="15">
         <v>40</v>
       </c>
@@ -4165,7 +4253,7 @@
         <v/>
       </c>
     </row>
-    <row r="41" ht="60" hidden="1" customHeight="1">
+    <row r="41" ht="60" customHeight="1">
       <c r="A41" s="15">
         <v>41</v>
       </c>
@@ -4213,7 +4301,7 @@
         <v/>
       </c>
     </row>
-    <row r="42" ht="60" hidden="1" customHeight="1">
+    <row r="42" ht="60" customHeight="1">
       <c r="A42" s="15">
         <v>42</v>
       </c>
@@ -4234,30 +4322,30 @@
         <v xml:space="preserve">(1) Hak-hak Subjek Data Pribadi sebagaimana dimaksud dalam Pasal 8, Pasal 9, Pasal 10 ayat (1), Pasal 11, dan Pasal 13 ayat (1) dan ayat (2) dikecualikan untuk:a. kepentingan pertahanan dan keamanan nasional; b. kepentingan proses penegakan hukum; c. kepentingan umum dalam rangka penyelenggaraan negara; d. kepentingan pengawasan sektor jasa keuangan, moneter, sistem pembayaran, dan stabilitas sistem keuangan yang dilakukan dalam rangka penyelenggaraan negara; atau e. kepentingan statistik dan penelitian ilmiah. (2) Pengecualian sebagaimana dimaksud pada ayat (1) dilaksanakan hanya dalam rangka pelaksanaan ketentuan Undang-Undang.</v>
       </c>
       <c r="F42" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="G42" s="18" t="s">
         <v>63</v>
       </c>
-      <c r="G42" s="18" t="s">
-        <v>83</v>
-      </c>
       <c r="H42" s="18" t="s">
+        <v>94</v>
+      </c>
+      <c r="I42" s="18" t="s">
+        <v>73</v>
+      </c>
+      <c r="J42" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="K42" s="18" t="s">
         <v>88</v>
       </c>
-      <c r="I42" s="18" t="s">
-        <v>66</v>
-      </c>
-      <c r="J42" s="18" t="s">
-        <v>67</v>
-      </c>
-      <c r="K42" s="18" t="s">
-        <v>89</v>
-      </c>
       <c r="L42" s="18" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="M42" s="19"/>
       <c r="N42" s="19"/>
       <c r="O42" s="15" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="P42" s="17" t="str">
         <f t="shared" si="2"/>
@@ -4277,7 +4365,7 @@
         <v/>
       </c>
     </row>
-    <row r="43" ht="60" hidden="1" customHeight="1">
+    <row r="43" ht="60" customHeight="1">
       <c r="A43" s="15">
         <v>43</v>
       </c>
@@ -4325,7 +4413,7 @@
         <v/>
       </c>
     </row>
-    <row r="44" ht="60" hidden="1" customHeight="1">
+    <row r="44" ht="60" customHeight="1">
       <c r="A44" s="15">
         <v>44</v>
       </c>
@@ -4346,30 +4434,30 @@
         <v xml:space="preserve">(1) Pemasangan alat pemroses atau pengolah data visual di tempat umum dan/ atau pada fasilitas pelayanan publik dilakukan dengan ketentuan: a. untuk tujuan keamanan, pencegahan bencana, lalu lintas atau dan/atau pengumpulan, analisis, dan pengaturan Informasi lalu lintas; b. harus menampilkan Informasi pada area yang telah dipasang alat pemroses atau pengolah data visual; dan c. tidak digunakan untuk seseorang. (2) Ketentuan sebagaimana dimaksud pada ayat (1) huruf b dan huruf c dikecualikan untuk pencegahan tindak pidana dan proses penegakan hukum sesuai dengan ketentuan peraturan perundang-undangan.</v>
       </c>
       <c r="F44" s="18" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="G44" s="18" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="H44" s="18" t="s">
+        <v>94</v>
+      </c>
+      <c r="I44" s="18" t="s">
+        <v>87</v>
+      </c>
+      <c r="J44" s="18" t="s">
+        <v>95</v>
+      </c>
+      <c r="K44" s="18" t="s">
         <v>88</v>
       </c>
-      <c r="I44" s="18" t="s">
-        <v>91</v>
-      </c>
-      <c r="J44" s="18" t="s">
-        <v>92</v>
-      </c>
-      <c r="K44" s="18" t="s">
-        <v>89</v>
-      </c>
       <c r="L44" s="18" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="M44" s="19"/>
       <c r="N44" s="19"/>
       <c r="O44" s="15" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="P44" s="17" t="str">
         <f t="shared" si="2"/>
@@ -4389,7 +4477,7 @@
         <v/>
       </c>
     </row>
-    <row r="45" ht="60" hidden="1" customHeight="1">
+    <row r="45" ht="60" customHeight="1">
       <c r="A45" s="15">
         <v>45</v>
       </c>
@@ -4437,7 +4525,7 @@
         <v/>
       </c>
     </row>
-    <row r="46" ht="60" hidden="1" customHeight="1">
+    <row r="46" ht="60" customHeight="1">
       <c r="A46" s="15">
         <v>46</v>
       </c>
@@ -4486,7 +4574,7 @@
 Umum</v>
       </c>
     </row>
-    <row r="47" ht="60" hidden="1" customHeight="1">
+    <row r="47" ht="60" customHeight="1">
       <c r="A47" s="15">
         <v>47</v>
       </c>
@@ -4534,7 +4622,7 @@
         <v xml:space="preserve">Bagian Kedua Kewajiban Pengendali Data Pribadi</v>
       </c>
     </row>
-    <row r="48" ht="60" hidden="1" customHeight="1">
+    <row r="48" ht="60" customHeight="1">
       <c r="A48" s="15">
         <v>48</v>
       </c>
@@ -4582,7 +4670,7 @@
         <v xml:space="preserve">Bagian Kedua Kewajiban Pengendali Data Pribadi</v>
       </c>
     </row>
-    <row r="49" ht="60" customHeight="1">
+    <row r="49" ht="140.25">
       <c r="A49" s="15">
         <v>49</v>
       </c>
@@ -4602,25 +4690,39 @@
         <f>IF(INDEX(Korpus!$F:$F,$A49)="","",INDEX(Korpus!$F:$F,$A49))</f>
         <v xml:space="preserve">(1) Persetujuan pemrosesan Data Pribadi dilakukan melalui persetujuan tertulis atau terekam. (2) Persetujuan sebagaimana dimaksud pada ayat (1) dapat disampaikan secara elektronik atau nonelektronik.(3) Persetujuan sebagaimana dimaksud pada ayat (1) mempunyai kekuatan hukum yang sama.(4). Dalam hal persetuluan sebagaimana dimaksud pada ayat (1) memuat tujuan lain, permintaan persetujuan harus memenuhi ketentuan:a. dapat dibedakan secara jelas dengan hal lainnya; b. dibuat dengan format yang dapat dipahami dan mudah diakses; dan c. menggunakan bahasa yang sederhana dan jelas.(5) Persetujuan yang tidak memenuhi ketentuan sebagaimana dimaksud pada ayat (1) dan ayat (4) dinyatakan batal demi hukum.</v>
       </c>
-      <c r="F49" s="18"/>
-      <c r="G49" s="18"/>
-      <c r="H49" s="18"/>
-      <c r="I49" s="18"/>
-      <c r="J49" s="18"/>
-      <c r="K49" s="18"/>
-      <c r="L49" s="18"/>
+      <c r="F49" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="G49" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="H49" s="18" t="s">
+        <v>97</v>
+      </c>
+      <c r="I49" s="18" t="s">
+        <v>83</v>
+      </c>
+      <c r="J49" s="18" t="s">
+        <v>98</v>
+      </c>
+      <c r="K49" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="L49" s="18" t="s">
+        <v>90</v>
+      </c>
       <c r="M49" s="19"/>
       <c r="N49" s="19"/>
       <c r="O49" s="15" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="P49" s="17" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve">Belum lengkap (6)</v>
+        <v>Lengkap</v>
       </c>
       <c r="Q49" s="17" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>OK</v>
       </c>
       <c r="R49" s="17" t="str">
         <f>IF(INDEX(Korpus!$B:$B,$A49)="","",INDEX(Korpus!$B:$B,$A49))</f>
@@ -4632,7 +4734,7 @@
         <v xml:space="preserve">Bagian Kedua Kewajiban Pengendali Data Pribadi</v>
       </c>
     </row>
-    <row r="50" ht="60" hidden="1" customHeight="1">
+    <row r="50" ht="60" customHeight="1">
       <c r="A50" s="15">
         <v>50</v>
       </c>
@@ -4680,7 +4782,7 @@
         <v xml:space="preserve">Bagian Kedua Kewajiban Pengendali Data Pribadi</v>
       </c>
     </row>
-    <row r="51" ht="60" hidden="1" customHeight="1">
+    <row r="51" ht="60" customHeight="1">
       <c r="A51" s="15">
         <v>51</v>
       </c>
@@ -4728,7 +4830,7 @@
         <v xml:space="preserve">Bagian Kedua Kewajiban Pengendali Data Pribadi</v>
       </c>
     </row>
-    <row r="52" ht="60" hidden="1" customHeight="1">
+    <row r="52" ht="60" customHeight="1">
       <c r="A52" s="15">
         <v>52</v>
       </c>
@@ -4749,22 +4851,22 @@
         <v xml:space="preserve">(1) Pemrosesan Data Pribadi anak secara khusus.(2) Pemrosesan Data Pribadi anak sebagaimana dimaksud pada ayat (1) wajib mendapat persetujuan dari orang tua anak dan/ atau wali anak sesuai dengan ketentuan peraturan perundang-undangan.</v>
       </c>
       <c r="F52" s="18" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="G52" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="H52" s="18" t="s">
+        <v>100</v>
+      </c>
+      <c r="I52" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="H52" s="18" t="s">
+      <c r="J52" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="I52" s="18" t="s">
-        <v>96</v>
-      </c>
-      <c r="J52" s="18" t="s">
-        <v>92</v>
-      </c>
       <c r="K52" s="18" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="L52" s="18" t="s">
         <v>97</v>
@@ -4772,7 +4874,7 @@
       <c r="M52" s="19"/>
       <c r="N52" s="19"/>
       <c r="O52" s="15" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="P52" s="17" t="str">
         <f t="shared" si="2"/>
@@ -4792,7 +4894,7 @@
         <v xml:space="preserve">Bagian Kedua Kewajiban Pengendali Data Pribadi</v>
       </c>
     </row>
-    <row r="53" ht="60" hidden="1" customHeight="1">
+    <row r="53" ht="100" customHeight="1">
       <c r="A53" s="15">
         <v>53</v>
       </c>
@@ -4840,7 +4942,7 @@
         <v xml:space="preserve">Bagian Kedua Kewajiban Pengendali Data Pribadi</v>
       </c>
     </row>
-    <row r="54" ht="60" hidden="1" customHeight="1">
+    <row r="54" ht="150" customHeight="1">
       <c r="A54" s="15">
         <v>54</v>
       </c>
@@ -4861,30 +4963,30 @@
         <v xml:space="preserve">Pengendali Data Pribadi wajib melakukan pemrosesan Data Pribadi secara terbatas dan spesifik, sah secara hukum, dan transparan.</v>
       </c>
       <c r="F54" s="18" t="s">
+        <v>101</v>
+      </c>
+      <c r="G54" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="H54" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="I54" s="18" t="s">
+        <v>83</v>
+      </c>
+      <c r="J54" s="18" t="s">
         <v>98</v>
       </c>
-      <c r="G54" s="18" t="s">
-        <v>83</v>
-      </c>
-      <c r="H54" s="18" t="s">
-        <v>69</v>
-      </c>
-      <c r="I54" s="18" t="s">
+      <c r="K54" s="18" t="s">
+        <v>88</v>
+      </c>
+      <c r="L54" s="18" t="s">
         <v>96</v>
-      </c>
-      <c r="J54" s="18" t="s">
-        <v>99</v>
-      </c>
-      <c r="K54" s="18" t="s">
-        <v>89</v>
-      </c>
-      <c r="L54" s="18" t="s">
-        <v>93</v>
       </c>
       <c r="M54" s="19"/>
       <c r="N54" s="19"/>
       <c r="O54" s="15" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="P54" s="17" t="str">
         <f t="shared" si="2"/>
@@ -4924,25 +5026,39 @@
         <f>IF(INDEX(Korpus!$F:$F,$A55)="","",INDEX(Korpus!$F:$F,$A55))</f>
         <v xml:space="preserve">Pengendali Data Pribadi wajib melakukan pemrosesan Data Pribadi sesuai dengan tujuan pemrosesan Data Pribadi.</v>
       </c>
-      <c r="F55" s="18"/>
-      <c r="G55" s="18"/>
-      <c r="H55" s="18"/>
-      <c r="I55" s="18"/>
-      <c r="J55" s="18"/>
-      <c r="K55" s="18"/>
-      <c r="L55" s="18"/>
+      <c r="F55" s="18" t="s">
+        <v>101</v>
+      </c>
+      <c r="G55" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="H55" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="I55" s="18" t="s">
+        <v>83</v>
+      </c>
+      <c r="J55" s="18" t="s">
+        <v>102</v>
+      </c>
+      <c r="K55" s="18" t="s">
+        <v>88</v>
+      </c>
+      <c r="L55" s="18" t="s">
+        <v>96</v>
+      </c>
       <c r="M55" s="19"/>
       <c r="N55" s="19"/>
       <c r="O55" s="15" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="P55" s="17" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve">Belum lengkap (6)</v>
+        <v>Lengkap</v>
       </c>
       <c r="Q55" s="17" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>OK</v>
       </c>
       <c r="R55" s="17" t="str">
         <f>IF(INDEX(Korpus!$B:$B,$A55)="","",INDEX(Korpus!$B:$B,$A55))</f>
@@ -4954,7 +5070,7 @@
         <v xml:space="preserve">Bagian Kedua Kewajiban Pengendali Data Pribadi</v>
       </c>
     </row>
-    <row r="56" ht="60" hidden="1" customHeight="1">
+    <row r="56" ht="60" customHeight="1">
       <c r="A56" s="15">
         <v>56</v>
       </c>
@@ -4975,30 +5091,30 @@
         <v xml:space="preserve">(1) Pengendali Data Pribadi wajib memastikan akurasi, kelengkapan, dan konsistensi Data Pribadi sesuai dengan ketentuan peraturan perundang-undangan.(2) Dalam memastikan akurasi, kelengkapan, dan konsistensi Data Pribadi sebagaimana dimaksud pada ayat (1) Pengendali Data Pribadi wajib melakukan verifikasi.</v>
       </c>
       <c r="F56" s="18" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="G56" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="H56" s="18" t="s">
+        <v>103</v>
+      </c>
+      <c r="I56" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="H56" s="18" t="s">
-        <v>100</v>
-      </c>
-      <c r="I56" s="18" t="s">
-        <v>96</v>
-      </c>
       <c r="J56" s="18" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="K56" s="18" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="L56" s="18" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="M56" s="19"/>
       <c r="N56" s="19"/>
       <c r="O56" s="15" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="P56" s="17" t="str">
         <f t="shared" si="2"/>
@@ -5018,7 +5134,7 @@
         <v xml:space="preserve">Bagian Kedua Kewajiban Pengendali Data Pribadi</v>
       </c>
     </row>
-    <row r="57" ht="60" hidden="1" customHeight="1">
+    <row r="57" ht="60" customHeight="1">
       <c r="A57" s="15">
         <v>57</v>
       </c>
@@ -5066,7 +5182,7 @@
         <v xml:space="preserve">Bagian Kedua Kewajiban Pengendali Data Pribadi</v>
       </c>
     </row>
-    <row r="58" ht="60" hidden="1" customHeight="1">
+    <row r="58" ht="60" customHeight="1">
       <c r="A58" s="15">
         <v>58</v>
       </c>
@@ -5114,7 +5230,7 @@
         <v xml:space="preserve">Bagian Kedua Kewajiban Pengendali Data Pribadi</v>
       </c>
     </row>
-    <row r="59" ht="60" hidden="1" customHeight="1">
+    <row r="59" ht="60" customHeight="1">
       <c r="A59" s="15">
         <v>59</v>
       </c>
@@ -5162,7 +5278,7 @@
         <v xml:space="preserve">Bagian Kedua Kewajiban Pengendali Data Pribadi</v>
       </c>
     </row>
-    <row r="60" ht="60" hidden="1" customHeight="1">
+    <row r="60" ht="60" customHeight="1">
       <c r="A60" s="15">
         <v>60</v>
       </c>
@@ -5210,7 +5326,7 @@
         <v xml:space="preserve">Bagian Kedua Kewajiban Pengendali Data Pribadi</v>
       </c>
     </row>
-    <row r="61" ht="60" hidden="1" customHeight="1">
+    <row r="61" ht="60" customHeight="1">
       <c r="A61" s="15">
         <v>61</v>
       </c>
@@ -5259,7 +5375,7 @@
 Kewajiban Pengendali Data Pribadi</v>
       </c>
     </row>
-    <row r="62" ht="60" customHeight="1">
+    <row r="62" ht="153">
       <c r="A62" s="15">
         <v>62</v>
       </c>
@@ -5279,25 +5395,39 @@
         <f>IF(INDEX(Korpus!$F:$F,$A62)="","",INDEX(Korpus!$F:$F,$A62))</f>
         <v xml:space="preserve">Pengendali Data Pribadi wajib melindungi dan memastikan keamanan Data Pribadi yang diprosesnya, dengan melakukan:a. penyusunan dan penerapan langkah teknis operasional untuk melindungi Data Pribadi dari gangguan pemrosesan Data Pribadi yang bertentangan dengan ketentuan peraturan perundang-undangan; dan b. penentuan tingkat keamanan Data Pribadi dengan memperhatikan sifat dan risiko dari Data Pribadi yang harus dilindungi dalam pemrosesan Data Pribadi.</v>
       </c>
-      <c r="F62" s="18"/>
-      <c r="G62" s="18"/>
-      <c r="H62" s="18"/>
-      <c r="I62" s="18"/>
-      <c r="J62" s="18"/>
-      <c r="K62" s="18"/>
-      <c r="L62" s="18"/>
+      <c r="F62" s="18" t="s">
+        <v>101</v>
+      </c>
+      <c r="G62" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="H62" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="I62" s="18" t="s">
+        <v>83</v>
+      </c>
+      <c r="J62" s="18" t="s">
+        <v>104</v>
+      </c>
+      <c r="K62" s="18" t="s">
+        <v>67</v>
+      </c>
+      <c r="L62" s="18" t="s">
+        <v>90</v>
+      </c>
       <c r="M62" s="19"/>
       <c r="N62" s="19"/>
       <c r="O62" s="15" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="P62" s="17" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve">Belum lengkap (6)</v>
+        <v>Lengkap</v>
       </c>
       <c r="Q62" s="17" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>OK</v>
       </c>
       <c r="R62" s="17" t="str">
         <f>IF(INDEX(Korpus!$B:$B,$A62)="","",INDEX(Korpus!$B:$B,$A62))</f>
@@ -5310,7 +5440,7 @@
 Kewajiban Pengendali Data Pribadi</v>
       </c>
     </row>
-    <row r="63" ht="60" hidden="1" customHeight="1">
+    <row r="63" ht="60" customHeight="1">
       <c r="A63" s="15">
         <v>63</v>
       </c>
@@ -5359,7 +5489,7 @@
 Kewajiban Pengendali Data Pribadi</v>
       </c>
     </row>
-    <row r="64" ht="60" hidden="1" customHeight="1">
+    <row r="64" ht="60" customHeight="1">
       <c r="A64" s="15">
         <v>64</v>
       </c>
@@ -5408,7 +5538,7 @@
 Kewajiban Pengendali Data Pribadi</v>
       </c>
     </row>
-    <row r="65" ht="60" hidden="1" customHeight="1">
+    <row r="65" ht="60" customHeight="1">
       <c r="A65" s="15">
         <v>65</v>
       </c>
@@ -5457,7 +5587,7 @@
 Kewajiban Pengendali Data Pribadi</v>
       </c>
     </row>
-    <row r="66" ht="60" hidden="1" customHeight="1">
+    <row r="66" ht="60" customHeight="1">
       <c r="A66" s="15">
         <v>66</v>
       </c>
@@ -5506,7 +5636,7 @@
 Kewajiban Pengendali Data Pribadi</v>
       </c>
     </row>
-    <row r="67" ht="60" customHeight="1">
+    <row r="67" ht="137.5">
       <c r="A67" s="15">
         <v>67</v>
       </c>
@@ -5526,25 +5656,39 @@
         <f>IF(INDEX(Korpus!$F:$F,$A67)="","",INDEX(Korpus!$F:$F,$A67))</f>
         <v xml:space="preserve">(1) Pengendali Data Pribadi wajib menghentikan pemrosesan Data Pribadi dalam hal Subjek Data Pribadi menarik kembali persetujuan pemrosesan Data Pribadi.(2) Penghentian pemrosesan Data Pribadi sebagaimana dimaksud pada ayat (1) dilakukan paling lambat 3 x 24 (tiga kali dua puluh empat) jam terhitung sejak Pengendali Data Pribadi menerima permintaan penarikan kembali persetujuan pemrosesan Data Pribadi.</v>
       </c>
-      <c r="F67" s="18"/>
-      <c r="G67" s="18"/>
-      <c r="H67" s="18"/>
-      <c r="I67" s="18"/>
-      <c r="J67" s="18"/>
-      <c r="K67" s="18"/>
-      <c r="L67" s="18"/>
+      <c r="F67" s="18" t="s">
+        <v>101</v>
+      </c>
+      <c r="G67" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="H67" s="18" t="s">
+        <v>97</v>
+      </c>
+      <c r="I67" s="18" t="s">
+        <v>83</v>
+      </c>
+      <c r="J67" s="18" t="s">
+        <v>93</v>
+      </c>
+      <c r="K67" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="L67" s="18" t="s">
+        <v>84</v>
+      </c>
       <c r="M67" s="19"/>
       <c r="N67" s="19"/>
       <c r="O67" s="15" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="P67" s="17" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve">Belum lengkap (6)</v>
+        <v>Lengkap</v>
       </c>
       <c r="Q67" s="17" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>OK</v>
       </c>
       <c r="R67" s="17" t="str">
         <f>IF(INDEX(Korpus!$B:$B,$A67)="","",INDEX(Korpus!$B:$B,$A67))</f>
@@ -5557,7 +5701,7 @@
 Kewajiban Pengendali Data Pribadi</v>
       </c>
     </row>
-    <row r="68" ht="60" hidden="1" customHeight="1">
+    <row r="68" ht="60" customHeight="1">
       <c r="A68" s="15">
         <v>68</v>
       </c>
@@ -5606,7 +5750,7 @@
 Kewajiban Pengendali Data Pribadi</v>
       </c>
     </row>
-    <row r="69" ht="60" hidden="1" customHeight="1">
+    <row r="69" ht="60" customHeight="1">
       <c r="A69" s="15">
         <v>69</v>
       </c>
@@ -5655,7 +5799,7 @@
 Kewajiban Pengendali Data Pribadi</v>
       </c>
     </row>
-    <row r="70" ht="60" hidden="1" customHeight="1">
+    <row r="70" ht="60" customHeight="1">
       <c r="A70" s="15">
         <v>70</v>
       </c>
@@ -5676,30 +5820,30 @@
         <v xml:space="preserve">(1) Pengendali Data Pribadi wajib menghapus Data Pribadi dalam hal:a. Data Pribadi tidak lagi diperlukan untuk pencapaian tujuan pemrosesan Data Pribadi; b. Subjek Data Pribadi telah melakukan penarikan kembali persetujuan pemrosesan Data Pribadi; c. terdapat permintaan dari Subjek Data Pribadi; atau d. Data Pribadi diperoleh dan/ atau diproses dengan cara melawan hukum.(2) Data Pribadi sebagaimana dimaksud pada ayat (1) dilakukan sesuai dengan ketentuan peraturan perundang-undangan.</v>
       </c>
       <c r="F70" s="18" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="G70" s="18" t="s">
-        <v>83</v>
+        <v>63</v>
       </c>
       <c r="H70" s="18" t="s">
         <v>84</v>
       </c>
       <c r="I70" s="18" t="s">
-        <v>96</v>
+        <v>83</v>
       </c>
       <c r="J70" s="18" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="K70" s="18" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="L70" s="18" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="M70" s="19"/>
       <c r="N70" s="19"/>
       <c r="O70" s="15" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="P70" s="17" t="str">
         <f t="shared" si="2"/>
@@ -5720,7 +5864,7 @@
 Kewajiban Pengendali Data Pribadi</v>
       </c>
     </row>
-    <row r="71" ht="60" hidden="1" customHeight="1">
+    <row r="71" ht="60" customHeight="1">
       <c r="A71" s="15">
         <v>71</v>
       </c>
@@ -5769,7 +5913,7 @@
 Kewajiban Pengendali Data Pribadi</v>
       </c>
     </row>
-    <row r="72" ht="60" hidden="1" customHeight="1">
+    <row r="72" ht="60" customHeight="1">
       <c r="A72" s="15">
         <v>72</v>
       </c>
@@ -5818,7 +5962,7 @@
 Kewajiban Pengendali Data Pribadi</v>
       </c>
     </row>
-    <row r="73" ht="60" hidden="1" customHeight="1">
+    <row r="73" ht="60" customHeight="1">
       <c r="A73" s="15">
         <v>73</v>
       </c>
@@ -5867,7 +6011,7 @@
 Kewajiban Pengendali Data Pribadi</v>
       </c>
     </row>
-    <row r="74" ht="60" hidden="1" customHeight="1">
+    <row r="74" ht="60" customHeight="1">
       <c r="A74" s="15">
         <v>74</v>
       </c>
@@ -5916,7 +6060,7 @@
 Kewajiban Pengendali Data Pribadi</v>
       </c>
     </row>
-    <row r="75" ht="60" hidden="1" customHeight="1">
+    <row r="75" ht="60" customHeight="1">
       <c r="A75" s="15">
         <v>75</v>
       </c>
@@ -5965,7 +6109,7 @@
 Kewajiban Pengendali Data Pribadi</v>
       </c>
     </row>
-    <row r="76" ht="60" hidden="1" customHeight="1">
+    <row r="76" ht="60" customHeight="1">
       <c r="A76" s="15">
         <v>76</v>
       </c>
@@ -6014,7 +6158,7 @@
 Kewajiban Pengendali Data Pribadi</v>
       </c>
     </row>
-    <row r="77" ht="60" hidden="1" customHeight="1">
+    <row r="77" ht="60" customHeight="1">
       <c r="A77" s="15">
         <v>77</v>
       </c>
@@ -6063,7 +6207,7 @@
 Kewajiban Pengendali Data Pribadi</v>
       </c>
     </row>
-    <row r="78" ht="60" hidden="1" customHeight="1">
+    <row r="78" ht="60" customHeight="1">
       <c r="A78" s="15">
         <v>78</v>
       </c>
@@ -6112,7 +6256,7 @@
 Kewajiban Prosesor Data Pribadi</v>
       </c>
     </row>
-    <row r="79" ht="60" hidden="1" customHeight="1">
+    <row r="79" ht="60" customHeight="1">
       <c r="A79" s="15">
         <v>79</v>
       </c>
@@ -6133,30 +6277,30 @@
         <v xml:space="preserve">Ketentuan mengenai kewajiban Pengendali Data Pribadi sebagaimana dimaksud dalam Pasal 29, Pasal 31, Pasal 35, Pasal 36, Pasal 37, Pasal 38, dan Pasal 39 berlaku juga terhadap Prosesor Data Pribadi.</v>
       </c>
       <c r="F79" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="G79" s="18" t="s">
         <v>63</v>
       </c>
-      <c r="G79" s="18" t="s">
-        <v>83</v>
-      </c>
       <c r="H79" s="18" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="I79" s="18" t="s">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="J79" s="18" t="s">
-        <v>81</v>
+        <v>66</v>
       </c>
       <c r="K79" s="18" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="L79" s="18" t="s">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="M79" s="19"/>
       <c r="N79" s="19"/>
       <c r="O79" s="15" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="P79" s="17" t="str">
         <f t="shared" si="4"/>
@@ -6177,7 +6321,7 @@
 Kewajiban Prosesor Data Pribadi</v>
       </c>
     </row>
-    <row r="80" ht="60" hidden="1" customHeight="1">
+    <row r="80" ht="60" customHeight="1">
       <c r="A80" s="15">
         <v>80</v>
       </c>
@@ -6226,7 +6370,7 @@
 Pejabat atau Petugas yang Melaksanakan Fungsi Pelindungan Data Pribadi</v>
       </c>
     </row>
-    <row r="81" ht="60" hidden="1" customHeight="1">
+    <row r="81" ht="60" customHeight="1">
       <c r="A81" s="15">
         <v>81</v>
       </c>
@@ -6247,30 +6391,30 @@
         <v xml:space="preserve">(1) Pengendali Data Pribadi dapat melakukan transfer Data Pribadi kepada Pengendali Data Pribadi lainnya dalam wilayah hukum Negara Republik Indonesia.(2) Pengendali Data Pribadi yang melakukan transfer Data Pribadi dan yang menerima transfer Data Pribadi wajib melakukan Pelindungan Data Pribadi sebagaimana dimaksud dalam Undang-Undang ini.</v>
       </c>
       <c r="F81" s="18" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="G81" s="18" t="s">
-        <v>83</v>
+        <v>63</v>
       </c>
       <c r="H81" s="18" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="I81" s="18" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="J81" s="18" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="K81" s="18" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="L81" s="18" t="s">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="M81" s="19"/>
       <c r="N81" s="19"/>
       <c r="O81" s="15" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="P81" s="17" t="str">
         <f t="shared" si="4"/>
@@ -6290,7 +6434,7 @@
 Transfer Data Pribadi Dalam Wilayah Hukum Negara Republik Indonesia</v>
       </c>
     </row>
-    <row r="82" ht="60" hidden="1" customHeight="1">
+    <row r="82" ht="60" customHeight="1">
       <c r="A82" s="15">
         <v>82</v>
       </c>
@@ -6337,7 +6481,7 @@
         <v xml:space="preserve">Bagian Kedua</v>
       </c>
     </row>
-    <row r="83" ht="60" customHeight="1">
+    <row r="83" ht="150">
       <c r="A83" s="15">
         <v>83</v>
       </c>
@@ -6357,25 +6501,39 @@
         <f>IF(INDEX(Korpus!$F:$F,$A83)="","",INDEX(Korpus!$F:$F,$A83))</f>
         <v xml:space="preserve">(1) Setiap Orang dilarang secara melawan hukum memperoleh atau mengumpulkan Data Pribadi yang bukan miliknya dengan maksud untuk menguntungkan diri sendiri atau orang lain yang dapat mengakibatkan kerugian Subjek Data Pribadi.(2) Setiap Orang dilarang secara melawan hukum mengungkapkan Data Pribadi yang bukan miliknya.(3) Setiap Orang dilarang secara melawan hukum menggunakan Data Pribadi yang bukan miliknya.</v>
       </c>
-      <c r="F83" s="18"/>
-      <c r="G83" s="18"/>
-      <c r="H83" s="18"/>
-      <c r="I83" s="18"/>
-      <c r="J83" s="18"/>
-      <c r="K83" s="18"/>
-      <c r="L83" s="18"/>
+      <c r="F83" s="18" t="s">
+        <v>99</v>
+      </c>
+      <c r="G83" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="H83" s="18" t="s">
+        <v>68</v>
+      </c>
+      <c r="I83" s="18" t="s">
+        <v>108</v>
+      </c>
+      <c r="J83" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="K83" s="18" t="s">
+        <v>88</v>
+      </c>
+      <c r="L83" s="18" t="s">
+        <v>64</v>
+      </c>
       <c r="M83" s="19"/>
       <c r="N83" s="19"/>
       <c r="O83" s="15" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="P83" s="17" t="str">
         <f t="shared" si="4"/>
-        <v xml:space="preserve">Belum lengkap (6)</v>
+        <v>Lengkap</v>
       </c>
       <c r="Q83" s="17" t="str">
         <f t="shared" si="5"/>
-        <v/>
+        <v>OK</v>
       </c>
       <c r="R83" s="17" t="str">
         <f>IF(INDEX(Korpus!$B:$B,$A83)="","",INDEX(Korpus!$B:$B,$A83))</f>
@@ -6387,7 +6545,7 @@
         <v/>
       </c>
     </row>
-    <row r="84" ht="60" hidden="1" customHeight="1">
+    <row r="84" ht="60" customHeight="1">
       <c r="A84" s="15">
         <v>84</v>
       </c>
@@ -6435,7 +6593,7 @@
         <v/>
       </c>
     </row>
-    <row r="85" ht="60" hidden="1" customHeight="1">
+    <row r="85" ht="60" customHeight="1">
       <c r="A85" s="15">
         <v>85</v>
       </c>
@@ -6503,25 +6661,39 @@
         <f>IF(INDEX(Korpus!$F:$F,$A86)="","",INDEX(Korpus!$F:$F,$A86))</f>
         <v xml:space="preserve">(1) Instansi Pusat dan Instansi Daerah mengakses Data di Portal Satu Data Indonesia tidak dipungut biaya.(2) Instansi Pusat dan Instansi Daerah dalam mengakses Data di Portal Satu Data Indonesia tidak memerlukan dokumen nota kesepahaman, perjanjian kerja sama, dan/atau dokumen surat pernyataan.</v>
       </c>
-      <c r="F86" s="18"/>
-      <c r="G86" s="18"/>
-      <c r="H86" s="18"/>
-      <c r="I86" s="18"/>
-      <c r="J86" s="18"/>
-      <c r="K86" s="18"/>
-      <c r="L86" s="18"/>
+      <c r="F86" s="18" t="s">
+        <v>109</v>
+      </c>
+      <c r="G86" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="H86" s="18" t="s">
+        <v>110</v>
+      </c>
+      <c r="I86" s="18" t="s">
+        <v>106</v>
+      </c>
+      <c r="J86" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="K86" s="18" t="s">
+        <v>88</v>
+      </c>
+      <c r="L86" s="18" t="s">
+        <v>94</v>
+      </c>
       <c r="M86" s="19"/>
       <c r="N86" s="19"/>
       <c r="O86" s="15" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="P86" s="17" t="str">
         <f t="shared" si="4"/>
-        <v xml:space="preserve">Belum lengkap (6)</v>
+        <v>Lengkap</v>
       </c>
       <c r="Q86" s="17" t="str">
         <f t="shared" si="5"/>
-        <v/>
+        <v>OK</v>
       </c>
       <c r="R86" s="17" t="str">
         <f>IF(INDEX(Korpus!$B:$B,$A86)="","",INDEX(Korpus!$B:$B,$A86))</f>
@@ -6535,13 +6707,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S86">
-    <filterColumn colId="14">
-      <filters>
-        <filter val="CC"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:S86"/>
   <dataValidations count="2" disablePrompts="0">
     <dataValidation sqref="M2:M86" type="none" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" prompt="Teks bebas, satu kalimat &quot;Sistem harus …&quot; atau “Sistem tidak boleh ...” (opsional, untuk R2)" showDropDown="0" showErrorMessage="1" showInputMessage="1"/>
     <dataValidation sqref="N2:N86" type="none" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" prompt="Digunakan untuk alasan T99, adanya keraguan, salah ketik atau teks terpotong, dan penjelasan lain bila aturan konsistensi tidak terpenuhi (Bagian 5.1 dan 9.1)." showDropDown="0" showErrorMessage="1" showInputMessage="1"/>
@@ -6605,7 +6771,7 @@
     </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="8" disablePrompts="0">
-        <x14:dataValidation xr:uid="{5AB987B5-8F3F-4A18-8FCD-1A01250F3F1E}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Kodekan pihak yang secara eksplisit menjadi subjek tata bahasa norma utama pada kolom “Isi”.&#10;Pilih kode berurutan dan berhenti pada Subjek Norma pertama yang dianggap sesuai (S1 &gt; S2 &gt; S3 &gt; S4 &gt; S5 &gt; S6 &gt; S7 &gt; S8 &gt; S9)." showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{49D78163-3F72-48B8-B1E8-456A6542C2F9}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Kodekan pihak yang secara eksplisit menjadi subjek tata bahasa norma utama pada kolom “Isi”.&#10;Pilih kode berurutan dan berhenti pada Subjek Norma pertama yang dianggap sesuai (S1 &gt; S2 &gt; S3 &gt; S4 &gt; S5 &gt; S6 &gt; S7 &gt; S8 &gt; S9)." showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>'Daftar Kode'!$D$5:$D$13</xm:f>
           </x14:formula1>
@@ -6614,7 +6780,7 @@
           </x14:formula2>
           <xm:sqref>F3:F86</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{6956030B-6D2B-46A8-B5E5-A9E353C50442}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Tentukan dengan Uji Implikasi Bagian 6." promptTitle="" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{3CA30908-FB0F-40C5-A8A4-F92F32DB696F}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Tentukan dengan Uji Implikasi Bagian 6." showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>'Daftar Kode'!$D$16:$D$18</xm:f>
           </x14:formula1>
@@ -6623,7 +6789,7 @@
           </x14:formula2>
           <xm:sqref>G2:G86</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{0235AB53-B601-4F0C-A78B-81CF67D714A8}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Pilih satu tema dominan dari pohon keputusan Bagian 7.3. Pemilihan T99 wajib dijelaskan di V12." showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{50CCF919-4331-4386-8595-79EA76AF6ACE}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Pilih satu tema dominan dari pohon keputusan Bagian 7.3. Pemilihan T99 wajib dijelaskan di V12." showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>'Daftar Kode'!$D$21:$D$37</xm:f>
           </x14:formula1>
@@ -6632,7 +6798,7 @@
           </x14:formula2>
           <xm:sqref>H2:H86</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{4D785A3B-70C9-48E7-9453-970154BC1193}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Lihat Bagian 7.4" promptTitle="" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{7CE5C7BE-2BCD-4E40-8077-B585E11BC8A3}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Lihat Bagian 7.4" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>'Daftar Kode'!$D$40:$D$47</xm:f>
           </x14:formula1>
@@ -6641,7 +6807,7 @@
           </x14:formula2>
           <xm:sqref>I2:I86</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{2C13D2DA-D41C-41BE-A982-016866542D6A}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Tahap siklus data yang terkait dari awal hingga akhir.&#10;Lihat Bagian 7.5" promptTitle="" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{4B666A14-D9D0-4FB3-9AD9-74AC08A78771}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Tahap siklus data yang terkait dari awal hingga akhir.&#10;Lihat Bagian 7.5" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>'Daftar Kode'!$D$50:$D$57</xm:f>
           </x14:formula1>
@@ -6650,7 +6816,7 @@
           </x14:formula2>
           <xm:sqref>J2:J86</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{2B5F0096-AB80-4B6C-9FA2-0BED7272C486}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Kandidat jenis kebutuhan SRS diperiksa berurutan K1 &gt; K2 &gt; K3 &gt; K4 &gt; K5. Lihat Bagian 7.6" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{58033816-4EA1-42A2-BB9D-361B87ADCAF2}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Kandidat jenis kebutuhan SRS diperiksa berurutan K1 &gt; K2 &gt; K3 &gt; K4 &gt; K5. Lihat Bagian 7.6" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>'Daftar Kode'!$D$60:$D$64</xm:f>
           </x14:formula1>
@@ -6659,7 +6825,7 @@
           </x14:formula2>
           <xm:sqref>K2:K86</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{65DDCB1A-04FF-4B4F-B401-52E603A7A314}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Tema kedua bila unit memuat dua tema (gunakan kode dari Bagian 7.3). T99 tidak digunakan di sini." promptTitle="Opsional" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{28FFE57B-0C89-4BBF-B3BC-007541E19009}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Tema kedua bila unit memuat dua tema (gunakan kode dari Bagian 7.3). T99 tidak digunakan di sini." promptTitle="Opsional" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>'Daftar Kode'!$D$21:$D$36</xm:f>
           </x14:formula1>
@@ -6668,7 +6834,7 @@
           </x14:formula2>
           <xm:sqref>L2:L86</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{2129703A-C87D-4D30-91F9-00316166868E}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Kodekan pihak yang secara eksplisit menjadi subjek tata bahasa norma utama pada kolom “Isi”. Jangan menyimpulkan subjek dari judul BAB." showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{7C010E85-4AA4-44D9-8E38-7D4EE486F56C}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Kodekan pihak yang secara eksplisit menjadi subjek tata bahasa norma utama pada kolom “Isi”. Jangan menyimpulkan subjek dari judul BAB." showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>'Daftar Kode'!$D$5:$D$13</xm:f>
           </x14:formula1>
@@ -6696,23 +6862,23 @@
   <sheetData>
     <row r="1" ht="18">
       <c r="A1" s="2" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="13" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="B4" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="D4" s="21" t="str">
         <f t="shared" ref="D4:D9" si="6">$B4 &amp; " - " &amp; $C4</f>
@@ -6724,10 +6890,10 @@
         <v>32</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="C5" s="22" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="D5" s="20" t="str">
         <f t="shared" si="6"/>
@@ -6739,10 +6905,10 @@
         <v>32</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="C6" s="22" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="D6" s="20" t="str">
         <f t="shared" si="6"/>
@@ -6754,10 +6920,10 @@
         <v>32</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="C7" s="22" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="D7" s="20" t="str">
         <f t="shared" si="6"/>
@@ -6769,10 +6935,10 @@
         <v>32</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="C8" s="22" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="D8" s="20" t="str">
         <f t="shared" si="6"/>
@@ -6784,10 +6950,10 @@
         <v>32</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="C9" s="22" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="D9" s="20" t="str">
         <f t="shared" si="6"/>
@@ -6799,10 +6965,10 @@
         <v>32</v>
       </c>
       <c r="B10" s="23" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="C10" s="22" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="D10" s="20" t="str">
         <f t="shared" ref="D10:D64" si="7">$B10 &amp; " - " &amp; $C10</f>
@@ -6814,10 +6980,10 @@
         <v>32</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="C11" s="22" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="D11" s="20" t="str">
         <f t="shared" si="7"/>
@@ -6829,10 +6995,10 @@
         <v>32</v>
       </c>
       <c r="B12" s="23" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="C12" s="22" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="D12" s="20" t="str">
         <f t="shared" si="7"/>
@@ -6844,10 +7010,10 @@
         <v>32</v>
       </c>
       <c r="B13" s="23" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="C13" s="22" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="D13" s="20" t="str">
         <f t="shared" si="7"/>
@@ -6856,13 +7022,13 @@
     </row>
     <row r="15">
       <c r="A15" s="13" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="B15" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="D15" s="21" t="str">
         <f t="shared" si="7"/>
@@ -6874,10 +7040,10 @@
         <v>34</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="C16" s="22" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="D16" s="20" t="str">
         <f t="shared" si="7"/>
@@ -6889,10 +7055,10 @@
         <v>34</v>
       </c>
       <c r="B17" s="23" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="C17" s="22" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="D17" s="20" t="str">
         <f t="shared" si="7"/>
@@ -6904,10 +7070,10 @@
         <v>34</v>
       </c>
       <c r="B18" s="23" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="C18" s="22" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="D18" s="20" t="str">
         <f t="shared" si="7"/>
@@ -6916,13 +7082,13 @@
     </row>
     <row r="20">
       <c r="A20" s="13" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="B20" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="D20" s="21" t="str">
         <f t="shared" si="7"/>
@@ -6934,10 +7100,10 @@
         <v>36</v>
       </c>
       <c r="B21" s="23" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="C21" s="22" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="D21" s="20" t="str">
         <f t="shared" si="7"/>
@@ -6949,10 +7115,10 @@
         <v>36</v>
       </c>
       <c r="B22" s="23" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="C22" s="22" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="D22" s="20" t="str">
         <f t="shared" si="7"/>
@@ -6964,10 +7130,10 @@
         <v>36</v>
       </c>
       <c r="B23" s="23" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="C23" s="22" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="D23" s="20" t="str">
         <f t="shared" si="7"/>
@@ -6979,10 +7145,10 @@
         <v>36</v>
       </c>
       <c r="B24" s="23" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="C24" s="22" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="D24" s="20" t="str">
         <f t="shared" si="7"/>
@@ -6994,10 +7160,10 @@
         <v>36</v>
       </c>
       <c r="B25" s="23" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="C25" s="22" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="D25" s="20" t="str">
         <f t="shared" si="7"/>
@@ -7009,10 +7175,10 @@
         <v>36</v>
       </c>
       <c r="B26" s="23" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="C26" s="22" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="D26" s="20" t="str">
         <f t="shared" si="7"/>
@@ -7024,10 +7190,10 @@
         <v>36</v>
       </c>
       <c r="B27" s="23" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="C27" s="22" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="D27" s="20" t="str">
         <f t="shared" si="7"/>
@@ -7039,10 +7205,10 @@
         <v>36</v>
       </c>
       <c r="B28" s="23" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="C28" s="22" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="D28" s="20" t="str">
         <f t="shared" si="7"/>
@@ -7054,10 +7220,10 @@
         <v>36</v>
       </c>
       <c r="B29" s="23" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="C29" s="22" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="D29" s="20" t="str">
         <f t="shared" si="7"/>
@@ -7069,10 +7235,10 @@
         <v>36</v>
       </c>
       <c r="B30" s="23" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="C30" s="22" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="D30" s="20" t="str">
         <f t="shared" si="7"/>
@@ -7084,10 +7250,10 @@
         <v>36</v>
       </c>
       <c r="B31" s="23" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="C31" s="22" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="D31" s="20" t="str">
         <f t="shared" si="7"/>
@@ -7099,10 +7265,10 @@
         <v>36</v>
       </c>
       <c r="B32" s="23" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="C32" s="22" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="D32" s="20" t="str">
         <f t="shared" si="7"/>
@@ -7114,10 +7280,10 @@
         <v>36</v>
       </c>
       <c r="B33" s="23" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="C33" s="22" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="D33" s="20" t="str">
         <f t="shared" si="7"/>
@@ -7129,10 +7295,10 @@
         <v>36</v>
       </c>
       <c r="B34" s="23" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="C34" s="22" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="D34" s="20" t="str">
         <f t="shared" si="7"/>
@@ -7144,10 +7310,10 @@
         <v>36</v>
       </c>
       <c r="B35" s="23" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="C35" s="22" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="D35" s="20" t="str">
         <f t="shared" si="7"/>
@@ -7159,10 +7325,10 @@
         <v>36</v>
       </c>
       <c r="B36" s="23" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="C36" s="22" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="D36" s="20" t="str">
         <f t="shared" si="7"/>
@@ -7174,10 +7340,10 @@
         <v>36</v>
       </c>
       <c r="B37" s="23" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="C37" s="22" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="D37" s="20" t="str">
         <f t="shared" si="7"/>
@@ -7186,13 +7352,13 @@
     </row>
     <row r="39">
       <c r="A39" s="13" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="B39" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C39" s="13" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="D39" s="21" t="str">
         <f t="shared" si="7"/>
@@ -7204,10 +7370,10 @@
         <v>38</v>
       </c>
       <c r="B40" s="23" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="C40" s="22" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="D40" s="20" t="str">
         <f t="shared" si="7"/>
@@ -7219,10 +7385,10 @@
         <v>38</v>
       </c>
       <c r="B41" s="23" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="C41" s="22" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="D41" s="20" t="str">
         <f t="shared" si="7"/>
@@ -7234,10 +7400,10 @@
         <v>38</v>
       </c>
       <c r="B42" s="23" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="C42" s="22" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="D42" s="20" t="str">
         <f t="shared" si="7"/>
@@ -7249,10 +7415,10 @@
         <v>38</v>
       </c>
       <c r="B43" s="23" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="C43" s="22" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="D43" s="20" t="str">
         <f t="shared" si="7"/>
@@ -7264,10 +7430,10 @@
         <v>38</v>
       </c>
       <c r="B44" s="23" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="C44" s="22" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="D44" s="20" t="str">
         <f t="shared" si="7"/>
@@ -7279,10 +7445,10 @@
         <v>38</v>
       </c>
       <c r="B45" s="23" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
       <c r="C45" s="22" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="D45" s="20" t="str">
         <f t="shared" si="7"/>
@@ -7294,10 +7460,10 @@
         <v>38</v>
       </c>
       <c r="B46" s="23" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="C46" s="22" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="D46" s="20" t="str">
         <f t="shared" si="7"/>
@@ -7309,10 +7475,10 @@
         <v>38</v>
       </c>
       <c r="B47" s="23" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="C47" s="22" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="D47" s="20" t="str">
         <f t="shared" si="7"/>
@@ -7321,13 +7487,13 @@
     </row>
     <row r="49">
       <c r="A49" s="13" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="B49" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C49" s="13" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="D49" s="21" t="str">
         <f t="shared" si="7"/>
@@ -7339,10 +7505,10 @@
         <v>40</v>
       </c>
       <c r="B50" s="23" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="C50" s="22" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="D50" s="20" t="str">
         <f t="shared" si="7"/>
@@ -7354,10 +7520,10 @@
         <v>40</v>
       </c>
       <c r="B51" s="23" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="C51" s="22" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
       <c r="D51" s="20" t="str">
         <f t="shared" si="7"/>
@@ -7369,10 +7535,10 @@
         <v>40</v>
       </c>
       <c r="B52" s="23" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="C52" s="22" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="D52" s="20" t="str">
         <f t="shared" si="7"/>
@@ -7384,10 +7550,10 @@
         <v>40</v>
       </c>
       <c r="B53" s="23" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="C53" s="22" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="D53" s="20" t="str">
         <f t="shared" si="7"/>
@@ -7399,10 +7565,10 @@
         <v>40</v>
       </c>
       <c r="B54" s="23" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="C54" s="22" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="D54" s="20" t="str">
         <f t="shared" si="7"/>
@@ -7414,10 +7580,10 @@
         <v>40</v>
       </c>
       <c r="B55" s="23" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="C55" s="22" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="D55" s="20" t="str">
         <f t="shared" si="7"/>
@@ -7429,10 +7595,10 @@
         <v>40</v>
       </c>
       <c r="B56" s="23" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="C56" s="22" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
       <c r="D56" s="20" t="str">
         <f t="shared" si="7"/>
@@ -7444,10 +7610,10 @@
         <v>40</v>
       </c>
       <c r="B57" s="23" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="C57" s="22" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="D57" s="20" t="str">
         <f t="shared" si="7"/>
@@ -7456,13 +7622,13 @@
     </row>
     <row r="59">
       <c r="A59" s="13" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="B59" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C59" s="13" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="D59" s="21" t="str">
         <f t="shared" si="7"/>
@@ -7474,10 +7640,10 @@
         <v>42</v>
       </c>
       <c r="B60" s="23" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="C60" s="22" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="D60" s="20" t="str">
         <f t="shared" si="7"/>
@@ -7489,10 +7655,10 @@
         <v>42</v>
       </c>
       <c r="B61" s="23" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="C61" s="22" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
       <c r="D61" s="20" t="str">
         <f t="shared" si="7"/>
@@ -7504,10 +7670,10 @@
         <v>42</v>
       </c>
       <c r="B62" s="23" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="C62" s="22" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
       <c r="D62" s="20" t="str">
         <f t="shared" si="7"/>
@@ -7519,10 +7685,10 @@
         <v>42</v>
       </c>
       <c r="B63" s="23" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="C63" s="22" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="D63" s="20" t="str">
         <f t="shared" si="7"/>
@@ -7534,10 +7700,10 @@
         <v>42</v>
       </c>
       <c r="B64" s="23" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="C64" s="22" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="D64" s="20" t="str">
         <f t="shared" si="7"/>
@@ -7567,7 +7733,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="24" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="B1" s="24" t="s">
         <v>60</v>
@@ -7576,1484 +7742,1484 @@
         <v>61</v>
       </c>
       <c r="D1" s="24" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="E1" s="24" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="F1" s="24" t="s">
         <v>56</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="B2" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C2" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="D2" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
       <c r="E2" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="F2" t="s">
-        <v>218</v>
+        <v>224</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="B3" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C3" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="D3" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
       <c r="E3" t="s">
-        <v>220</v>
+        <v>226</v>
       </c>
       <c r="F3" t="s">
-        <v>221</v>
+        <v>227</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>222</v>
+        <v>228</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="B4" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C4" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="D4" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
       <c r="E4" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="F4" t="s">
-        <v>224</v>
+        <v>230</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="B5" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C5" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="D5" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
       <c r="E5" t="s">
-        <v>226</v>
+        <v>232</v>
       </c>
       <c r="F5" t="s">
-        <v>227</v>
+        <v>233</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="B6" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C6" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="D6" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
       <c r="E6" t="s">
-        <v>228</v>
+        <v>234</v>
       </c>
       <c r="F6" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="B7" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C7" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="D7" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
       <c r="E7" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
       <c r="F7" t="s">
-        <v>231</v>
+        <v>237</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="B8" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C8" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="D8" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
       <c r="E8" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="F8" t="s">
-        <v>233</v>
+        <v>239</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="B9" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C9" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="D9" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
       <c r="E9" t="s">
-        <v>220</v>
+        <v>226</v>
       </c>
       <c r="F9" t="s">
-        <v>234</v>
+        <v>240</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="B10" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C10" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="D10" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
       <c r="E10" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="F10" t="s">
-        <v>235</v>
+        <v>241</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="B11" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C11" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="D11" t="s">
+        <v>238</v>
+      </c>
+      <c r="E11" t="s">
         <v>232</v>
       </c>
-      <c r="E11" t="s">
-        <v>226</v>
-      </c>
       <c r="F11" t="s">
-        <v>236</v>
+        <v>242</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="B12" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C12" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="D12" t="s">
-        <v>237</v>
+        <v>243</v>
       </c>
       <c r="E12" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="F12" t="s">
-        <v>238</v>
+        <v>244</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="B13" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C13" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="D13" t="s">
-        <v>237</v>
+        <v>243</v>
       </c>
       <c r="E13" t="s">
-        <v>220</v>
+        <v>226</v>
       </c>
       <c r="F13" t="s">
-        <v>239</v>
+        <v>245</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="B14" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C14" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="D14" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
       <c r="E14" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="F14" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="B15" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C15" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="D15" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
       <c r="E15" t="s">
-        <v>220</v>
+        <v>226</v>
       </c>
       <c r="F15" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="B16" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C16" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="D16" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
       <c r="E16" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="F16" t="s">
-        <v>243</v>
+        <v>249</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="B17" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C17" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="D17" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
       <c r="E17" t="s">
-        <v>244</v>
+        <v>250</v>
       </c>
       <c r="F17" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="B18" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C18" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="D18" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
       <c r="E18" t="s">
-        <v>246</v>
+        <v>252</v>
       </c>
       <c r="F18" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="B19" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C19" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="D19" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
       <c r="E19" t="s">
-        <v>248</v>
+        <v>254</v>
       </c>
       <c r="F19" t="s">
-        <v>249</v>
+        <v>255</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="B20" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C20" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="D20" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="E20" t="s">
-        <v>220</v>
+        <v>226</v>
       </c>
       <c r="F20" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="B21" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C21" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="D21" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="E21" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="F21" t="s">
-        <v>252</v>
+        <v>258</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="B22" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C22" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="D22" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="E22" t="s">
-        <v>226</v>
+        <v>232</v>
       </c>
       <c r="F22" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="B23" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C23" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="D23" t="s">
-        <v>254</v>
+        <v>260</v>
       </c>
       <c r="E23" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="F23" t="s">
-        <v>255</v>
+        <v>261</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="B24" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C24" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="D24" t="s">
-        <v>254</v>
+        <v>260</v>
       </c>
       <c r="E24" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="F24" t="s">
-        <v>256</v>
+        <v>262</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="B25" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="D25" t="s">
-        <v>258</v>
+        <v>264</v>
       </c>
       <c r="E25" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="F25" t="s">
-        <v>259</v>
+        <v>265</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="B26" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="D26" t="s">
-        <v>258</v>
+        <v>264</v>
       </c>
       <c r="E26" t="s">
-        <v>226</v>
+        <v>232</v>
       </c>
       <c r="F26" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
     </row>
     <row r="27" ht="58">
       <c r="A27" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>262</v>
+        <v>268</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
       <c r="E27" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="F27" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
     </row>
     <row r="28" ht="58">
       <c r="A28" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B28" s="11" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="E28" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="F28" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="29" ht="58">
       <c r="A29" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B29" s="11" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="E29" t="s">
-        <v>270</v>
+        <v>276</v>
       </c>
       <c r="F29" t="s">
-        <v>271</v>
+        <v>277</v>
       </c>
     </row>
     <row r="30" ht="29">
       <c r="A30" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B30" s="11" t="s">
-        <v>272</v>
+        <v>278</v>
       </c>
       <c r="E30" t="s">
-        <v>273</v>
+        <v>279</v>
       </c>
       <c r="F30" t="s">
-        <v>274</v>
+        <v>280</v>
       </c>
     </row>
     <row r="31" ht="58">
       <c r="A31" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B31" s="11" t="s">
-        <v>275</v>
+        <v>281</v>
       </c>
       <c r="E31" t="s">
-        <v>276</v>
+        <v>282</v>
       </c>
       <c r="F31" t="s">
-        <v>277</v>
+        <v>283</v>
       </c>
     </row>
     <row r="32" ht="72.5">
       <c r="A32" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B32" s="11" t="s">
-        <v>278</v>
+        <v>284</v>
       </c>
       <c r="E32" t="s">
-        <v>279</v>
+        <v>285</v>
       </c>
       <c r="F32" t="s">
-        <v>280</v>
+        <v>286</v>
       </c>
     </row>
     <row r="33" ht="72.5">
       <c r="A33" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B33" s="11" t="s">
-        <v>278</v>
+        <v>284</v>
       </c>
       <c r="E33" t="s">
-        <v>281</v>
+        <v>287</v>
       </c>
       <c r="F33" t="s">
-        <v>282</v>
+        <v>288</v>
       </c>
     </row>
     <row r="34" ht="72.5">
       <c r="A34" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B34" s="11" t="s">
-        <v>278</v>
+        <v>284</v>
       </c>
       <c r="E34" t="s">
-        <v>283</v>
+        <v>289</v>
       </c>
       <c r="F34" t="s">
-        <v>284</v>
+        <v>290</v>
       </c>
     </row>
     <row r="35" ht="72.5">
       <c r="A35" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B35" s="11" t="s">
-        <v>278</v>
+        <v>284</v>
       </c>
       <c r="E35" t="s">
-        <v>285</v>
+        <v>291</v>
       </c>
       <c r="F35" t="s">
-        <v>286</v>
+        <v>292</v>
       </c>
     </row>
     <row r="36" ht="72.5">
       <c r="A36" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B36" s="11" t="s">
-        <v>278</v>
+        <v>284</v>
       </c>
       <c r="E36" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="F36" t="s">
-        <v>288</v>
+        <v>294</v>
       </c>
     </row>
     <row r="37" ht="72.5">
       <c r="A37" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B37" s="11" t="s">
-        <v>278</v>
+        <v>284</v>
       </c>
       <c r="E37" t="s">
-        <v>289</v>
+        <v>295</v>
       </c>
       <c r="F37" t="s">
-        <v>290</v>
+        <v>296</v>
       </c>
     </row>
     <row r="38" ht="72.5">
       <c r="A38" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B38" s="11" t="s">
-        <v>278</v>
+        <v>284</v>
       </c>
       <c r="E38" t="s">
-        <v>291</v>
+        <v>297</v>
       </c>
       <c r="F38" t="s">
-        <v>292</v>
+        <v>298</v>
       </c>
     </row>
     <row r="39" ht="72.5">
       <c r="A39" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B39" s="11" t="s">
-        <v>278</v>
+        <v>284</v>
       </c>
       <c r="E39" t="s">
-        <v>293</v>
+        <v>299</v>
       </c>
       <c r="F39" t="s">
-        <v>294</v>
+        <v>300</v>
       </c>
     </row>
     <row r="40" ht="72.5">
       <c r="A40" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B40" s="11" t="s">
-        <v>278</v>
+        <v>284</v>
       </c>
       <c r="E40" t="s">
-        <v>295</v>
+        <v>301</v>
       </c>
       <c r="F40" t="s">
-        <v>296</v>
+        <v>302</v>
       </c>
     </row>
     <row r="41" ht="72.5">
       <c r="A41" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B41" s="11" t="s">
-        <v>278</v>
+        <v>284</v>
       </c>
       <c r="E41" t="s">
-        <v>297</v>
+        <v>303</v>
       </c>
       <c r="F41" t="s">
-        <v>298</v>
+        <v>304</v>
       </c>
     </row>
     <row r="42" ht="72.5">
       <c r="A42" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B42" s="11" t="s">
-        <v>278</v>
+        <v>284</v>
       </c>
       <c r="E42" t="s">
-        <v>299</v>
+        <v>305</v>
       </c>
       <c r="F42" t="s">
-        <v>300</v>
+        <v>306</v>
       </c>
     </row>
     <row r="43" ht="72.5">
       <c r="A43" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B43" s="11" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
       <c r="E43" t="s">
-        <v>302</v>
+        <v>308</v>
       </c>
       <c r="F43" t="s">
-        <v>303</v>
+        <v>309</v>
       </c>
     </row>
     <row r="44" ht="72.5">
       <c r="A44" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B44" s="11" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
       <c r="E44" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="F44" t="s">
-        <v>305</v>
+        <v>311</v>
       </c>
     </row>
     <row r="45" ht="72.5">
       <c r="A45" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B45" s="11" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
       <c r="E45" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
       <c r="F45" t="s">
-        <v>307</v>
+        <v>313</v>
       </c>
     </row>
     <row r="46" ht="232">
       <c r="A46" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B46" s="11" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C46" s="11" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="E46" t="s">
-        <v>310</v>
+        <v>316</v>
       </c>
       <c r="F46" t="s">
-        <v>311</v>
+        <v>317</v>
       </c>
     </row>
     <row r="47" ht="232">
       <c r="A47" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B47" s="11" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C47" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="E47" t="s">
-        <v>313</v>
+        <v>319</v>
       </c>
       <c r="F47" t="s">
-        <v>314</v>
+        <v>320</v>
       </c>
     </row>
     <row r="48" ht="232">
       <c r="A48" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B48" s="11" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C48" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="E48" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
       <c r="F48" t="s">
-        <v>316</v>
+        <v>322</v>
       </c>
     </row>
     <row r="49" ht="232">
       <c r="A49" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B49" s="11" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C49" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="E49" t="s">
-        <v>317</v>
+        <v>323</v>
       </c>
       <c r="F49" t="s">
-        <v>318</v>
+        <v>324</v>
       </c>
     </row>
     <row r="50" ht="232">
       <c r="A50" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B50" s="11" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C50" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="E50" t="s">
-        <v>319</v>
+        <v>325</v>
       </c>
       <c r="F50" t="s">
-        <v>320</v>
+        <v>326</v>
       </c>
     </row>
     <row r="51" ht="232">
       <c r="A51" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B51" s="11" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C51" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="E51" t="s">
-        <v>321</v>
+        <v>327</v>
       </c>
       <c r="F51" t="s">
-        <v>322</v>
+        <v>328</v>
       </c>
     </row>
     <row r="52" ht="232">
       <c r="A52" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B52" s="11" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C52" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="E52" t="s">
-        <v>323</v>
+        <v>329</v>
       </c>
       <c r="F52" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
     </row>
     <row r="53" ht="232">
       <c r="A53" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B53" s="11" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C53" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="E53" t="s">
-        <v>325</v>
+        <v>331</v>
       </c>
       <c r="F53" t="s">
-        <v>326</v>
+        <v>332</v>
       </c>
     </row>
     <row r="54" ht="232">
       <c r="A54" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B54" s="11" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C54" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="E54" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="F54" t="s">
-        <v>327</v>
+        <v>333</v>
       </c>
     </row>
     <row r="55" ht="232">
       <c r="A55" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B55" s="11" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C55" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="E55" t="s">
-        <v>328</v>
+        <v>334</v>
       </c>
       <c r="F55" t="s">
-        <v>329</v>
+        <v>335</v>
       </c>
     </row>
     <row r="56" ht="232">
       <c r="A56" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B56" s="11" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C56" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="E56" t="s">
-        <v>330</v>
+        <v>336</v>
       </c>
       <c r="F56" t="s">
-        <v>331</v>
+        <v>337</v>
       </c>
     </row>
     <row r="57" ht="232">
       <c r="A57" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B57" s="11" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C57" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="E57" t="s">
-        <v>332</v>
+        <v>338</v>
       </c>
       <c r="F57" t="s">
-        <v>333</v>
+        <v>339</v>
       </c>
     </row>
     <row r="58" ht="232">
       <c r="A58" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B58" s="11" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C58" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="E58" t="s">
-        <v>334</v>
+        <v>340</v>
       </c>
       <c r="F58" t="s">
-        <v>335</v>
+        <v>341</v>
       </c>
     </row>
     <row r="59" ht="232">
       <c r="A59" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B59" s="11" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C59" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="E59" t="s">
-        <v>336</v>
+        <v>342</v>
       </c>
       <c r="F59" t="s">
-        <v>337</v>
+        <v>343</v>
       </c>
     </row>
     <row r="60" ht="232">
       <c r="A60" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B60" s="11" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C60" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="E60" t="s">
-        <v>338</v>
+        <v>344</v>
       </c>
       <c r="F60" t="s">
-        <v>339</v>
+        <v>345</v>
       </c>
     </row>
     <row r="61" ht="232">
       <c r="A61" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B61" s="11" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C61" s="11" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="E61" t="s">
-        <v>341</v>
+        <v>347</v>
       </c>
       <c r="F61" t="s">
-        <v>342</v>
+        <v>348</v>
       </c>
     </row>
     <row r="62" ht="232">
       <c r="A62" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B62" s="11" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C62" s="11" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="E62" t="s">
-        <v>343</v>
+        <v>349</v>
       </c>
       <c r="F62" t="s">
-        <v>344</v>
+        <v>350</v>
       </c>
     </row>
     <row r="63" ht="232">
       <c r="A63" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B63" s="11" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C63" s="11" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="E63" t="s">
-        <v>345</v>
+        <v>351</v>
       </c>
       <c r="F63" t="s">
-        <v>346</v>
+        <v>352</v>
       </c>
     </row>
     <row r="64" ht="232">
       <c r="A64" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B64" s="11" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C64" s="11" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="E64" t="s">
-        <v>347</v>
+        <v>353</v>
       </c>
       <c r="F64" t="s">
-        <v>348</v>
+        <v>354</v>
       </c>
     </row>
     <row r="65" ht="232">
       <c r="A65" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B65" s="11" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C65" s="11" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="E65" t="s">
-        <v>349</v>
+        <v>355</v>
       </c>
       <c r="F65" t="s">
-        <v>350</v>
+        <v>356</v>
       </c>
     </row>
     <row r="66" ht="232">
       <c r="A66" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B66" s="11" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C66" s="11" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="E66" t="s">
-        <v>351</v>
+        <v>357</v>
       </c>
       <c r="F66" t="s">
-        <v>352</v>
+        <v>358</v>
       </c>
     </row>
     <row r="67" ht="232">
       <c r="A67" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B67" s="11" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C67" s="11" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="E67" t="s">
-        <v>353</v>
+        <v>359</v>
       </c>
       <c r="F67" t="s">
-        <v>354</v>
+        <v>360</v>
       </c>
     </row>
     <row r="68" ht="232">
       <c r="A68" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B68" s="11" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C68" s="11" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="E68" t="s">
-        <v>355</v>
+        <v>361</v>
       </c>
       <c r="F68" t="s">
-        <v>356</v>
+        <v>362</v>
       </c>
     </row>
     <row r="69" ht="232">
       <c r="A69" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B69" s="11" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C69" s="11" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="E69" t="s">
-        <v>357</v>
+        <v>363</v>
       </c>
       <c r="F69" t="s">
-        <v>358</v>
+        <v>364</v>
       </c>
     </row>
     <row r="70" ht="232">
       <c r="A70" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B70" s="11" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C70" s="11" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="E70" t="s">
-        <v>359</v>
+        <v>365</v>
       </c>
       <c r="F70" t="s">
-        <v>360</v>
+        <v>366</v>
       </c>
     </row>
     <row r="71" ht="232">
       <c r="A71" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B71" s="11" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C71" s="11" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="E71" t="s">
-        <v>361</v>
+        <v>367</v>
       </c>
       <c r="F71" t="s">
-        <v>362</v>
+        <v>368</v>
       </c>
     </row>
     <row r="72" ht="232">
       <c r="A72" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B72" s="11" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C72" s="11" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="E72" t="s">
-        <v>363</v>
+        <v>369</v>
       </c>
       <c r="F72" t="s">
-        <v>364</v>
+        <v>370</v>
       </c>
     </row>
     <row r="73" ht="232">
       <c r="A73" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B73" s="11" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C73" s="11" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="E73" t="s">
-        <v>365</v>
+        <v>371</v>
       </c>
       <c r="F73" t="s">
-        <v>366</v>
+        <v>372</v>
       </c>
     </row>
     <row r="74" ht="232">
       <c r="A74" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B74" s="11" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C74" s="11" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="E74" t="s">
-        <v>367</v>
+        <v>373</v>
       </c>
       <c r="F74" t="s">
-        <v>368</v>
+        <v>374</v>
       </c>
     </row>
     <row r="75" ht="232">
       <c r="A75" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B75" s="11" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C75" s="11" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="E75" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
       <c r="F75" t="s">
-        <v>370</v>
+        <v>376</v>
       </c>
     </row>
     <row r="76" ht="232">
       <c r="A76" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B76" s="11" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C76" s="11" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="E76" t="s">
-        <v>371</v>
+        <v>377</v>
       </c>
       <c r="F76" t="s">
-        <v>372</v>
+        <v>378</v>
       </c>
     </row>
     <row r="77" ht="232">
       <c r="A77" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B77" s="11" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C77" s="11" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="E77" t="s">
-        <v>373</v>
+        <v>379</v>
       </c>
       <c r="F77" t="s">
-        <v>374</v>
+        <v>380</v>
       </c>
     </row>
     <row r="78" ht="232">
       <c r="A78" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B78" s="11" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C78" s="11" t="s">
-        <v>375</v>
+        <v>381</v>
       </c>
       <c r="E78" t="s">
-        <v>376</v>
+        <v>382</v>
       </c>
       <c r="F78" s="25" t="s">
-        <v>377</v>
+        <v>383</v>
       </c>
     </row>
     <row r="79" ht="232">
       <c r="A79" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B79" s="11" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C79" s="11" t="s">
-        <v>375</v>
+        <v>381</v>
       </c>
       <c r="E79" t="s">
-        <v>378</v>
+        <v>384</v>
       </c>
       <c r="F79" t="s">
-        <v>379</v>
+        <v>385</v>
       </c>
     </row>
     <row r="80" ht="232">
       <c r="A80" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B80" s="11" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C80" s="11" t="s">
-        <v>380</v>
+        <v>386</v>
       </c>
       <c r="E80" t="s">
-        <v>381</v>
+        <v>387</v>
       </c>
       <c r="F80" t="s">
-        <v>382</v>
+        <v>388</v>
       </c>
     </row>
     <row r="81" ht="174">
       <c r="A81" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B81" t="s">
-        <v>383</v>
+        <v>389</v>
       </c>
       <c r="C81" s="11" t="s">
-        <v>384</v>
+        <v>390</v>
       </c>
       <c r="E81" t="s">
-        <v>385</v>
+        <v>391</v>
       </c>
       <c r="F81" t="s">
-        <v>386</v>
+        <v>392</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B82" t="s">
-        <v>383</v>
+        <v>389</v>
       </c>
       <c r="C82" t="s">
-        <v>387</v>
+        <v>393</v>
       </c>
       <c r="E82" t="s">
-        <v>388</v>
+        <v>394</v>
       </c>
       <c r="F82" t="s">
-        <v>389</v>
+        <v>395</v>
       </c>
     </row>
     <row r="83" ht="116">
       <c r="A83" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B83" s="11" t="s">
-        <v>390</v>
+        <v>396</v>
       </c>
       <c r="E83" t="s">
-        <v>391</v>
+        <v>397</v>
       </c>
       <c r="F83" t="s">
-        <v>392</v>
+        <v>398</v>
       </c>
     </row>
     <row r="84" ht="116">
       <c r="A84" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B84" s="11" t="s">
-        <v>390</v>
+        <v>396</v>
       </c>
       <c r="E84" t="s">
-        <v>393</v>
+        <v>399</v>
       </c>
       <c r="F84" t="s">
-        <v>394</v>
+        <v>400</v>
       </c>
     </row>
     <row r="85" ht="58">
       <c r="A85" t="s">
-        <v>395</v>
+        <v>401</v>
       </c>
       <c r="B85" s="11" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="E85" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="F85" t="s">
-        <v>396</v>
+        <v>402</v>
       </c>
     </row>
     <row r="86" ht="101.5">
       <c r="A86" t="s">
-        <v>395</v>
+        <v>401</v>
       </c>
       <c r="B86" s="11" t="s">
-        <v>397</v>
+        <v>403</v>
       </c>
       <c r="C86" s="11" t="s">
-        <v>398</v>
+        <v>404</v>
       </c>
       <c r="E86" t="s">
-        <v>351</v>
+        <v>357</v>
       </c>
       <c r="F86" t="s">
-        <v>399</v>
+        <v>405</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>400</v>
+        <v>406</v>
       </c>
       <c r="B87" t="s">
-        <v>401</v>
+        <v>407</v>
       </c>
     </row>
   </sheetData>

</xml_diff>